<commit_message>
Revision of leaf phenology and primary growth determinacy
</commit_message>
<xml_diff>
--- a/data-raw/SpParamsDefinition.xlsx
+++ b/data-raw/SpParamsDefinition.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="784" uniqueCount="388">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="789" uniqueCount="390">
   <si>
     <t xml:space="preserve">ParameterName</t>
   </si>
@@ -139,7 +139,13 @@
     <t xml:space="preserve">PhenologyType</t>
   </si>
   <si>
-    <t xml:space="preserve">Leaf phenology type, either "oneflush-evergreen" (new leaves develop in spring-summer), "progressive-evergreen" (new leaves develop during any season), "winter-deciduous" (leaf senescence in autumn, new leaves in spring-summer) or "winter-semideciduous" (same as before, but abscission of senescent leaves occurs when new leaves are produced).</t>
+    <t xml:space="preserve">Leaf phenology type, either "evergreen" , "winter-deciduous"  or "winter-semideciduous".</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GrowthDeterminacy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Growth determinacy type, either “determinate”, “indeterminate” or “intermediate”</t>
   </si>
   <si>
     <t xml:space="preserve">DispersalType</t>
@@ -911,35 +917,7 @@
     <t xml:space="preserve">VCleaf_kmax</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Maximum </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">whole-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">leaf hydraulic conductance</t>
-    </r>
+    <t xml:space="preserve">Maximum whole-leaf hydraulic conductance</t>
   </si>
   <si>
     <r>
@@ -1037,69 +1015,13 @@
     <t xml:space="preserve">VCleaf_P50</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">50% of maximum conductance of the </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">whole-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">leaf vulnerability curve</t>
-    </r>
+    <t xml:space="preserve">50% of maximum conductance of the whole-leaf vulnerability curve</t>
   </si>
   <si>
     <t xml:space="preserve">VCleaf_P88</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">88% of maximum conductance of the </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">whole-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">leaf vulnerability curve</t>
-    </r>
+    <t xml:space="preserve">88% of maximum conductance of the whole-leaf vulnerability curve</t>
   </si>
   <si>
     <t xml:space="preserve">VCleaf_slope</t>
@@ -1117,69 +1039,13 @@
     <t xml:space="preserve">VCleafapo_P50</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">50% of maximum conductance of the </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">leaf apoplasm</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve"> vulnerability curve</t>
-    </r>
+    <t xml:space="preserve">50% of maximum conductance of the leaf apoplasm vulnerability curve</t>
   </si>
   <si>
     <t xml:space="preserve">VCleafapo_P88</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">88% of maximum conductance of the </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">leaf apoplasm</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve"> vulnerability curve</t>
-    </r>
+    <t xml:space="preserve">88% of maximum conductance of the leaf apoplasm vulnerability curve</t>
   </si>
   <si>
     <t xml:space="preserve">VCleafapo_slope</t>
@@ -1553,7 +1419,7 @@
     <t xml:space="preserve">RGRleafmax</t>
   </si>
   <si>
-    <t xml:space="preserve">Maximum leaf relative growth rate</t>
+    <t xml:space="preserve">Maximum leaf growth rate relative to sapwood area</t>
   </si>
   <si>
     <t xml:space="preserve">m2/cm2/day</t>
@@ -1798,7 +1664,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="_-* #,##0.00\ _€_-;\-* #,##0.00\ _€_-;_-* \-??\ _€_-;_-@_-"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="10">
     <font>
       <sz val="12"/>
       <color rgb="FF000000"/>
@@ -1866,12 +1732,6 @@
       <name val="Symbol"/>
       <family val="1"/>
       <charset val="2"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -2095,7 +1955,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H164"/>
+  <dimension ref="A1:H1048576"/>
   <sheetFormatPr defaultColWidth="10.25" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="25.25"/>
@@ -2372,7 +2232,7 @@
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="1" t="s">
+      <c r="A15" s="3" t="s">
         <v>40</v>
       </c>
       <c r="B15" s="3" t="s">
@@ -2388,47 +2248,44 @@
         <v>31</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="3" t="s">
+      <c r="A16" s="1" t="s">
         <v>42</v>
       </c>
       <c r="B16" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C16" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="C16" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>45</v>
+      <c r="D16" s="5" t="s">
+        <v>11</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>46</v>
+        <v>31</v>
       </c>
       <c r="F16" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="G16" s="1" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C17" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E17" s="5" t="s">
         <v>48</v>
-      </c>
-      <c r="D17" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E17" s="5" t="s">
-        <v>46</v>
       </c>
       <c r="F17" s="1" t="n">
         <v>1</v>
@@ -2442,19 +2299,19 @@
         <v>49</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C18" s="1" t="s">
         <v>50</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="F18" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G18" s="1" t="n">
         <v>0</v>
@@ -2465,16 +2322,16 @@
         <v>51</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C19" s="1" t="s">
         <v>52</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="F19" s="1" t="n">
         <v>0</v>
@@ -2485,22 +2342,22 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="C20" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="B20" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="C20" s="1" t="s">
+      <c r="D20" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E20" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="D20" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E20" s="5" t="s">
-        <v>53</v>
-      </c>
       <c r="F20" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G20" s="1" t="n">
         <v>0</v>
@@ -2511,17 +2368,19 @@
         <v>56</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C21" s="1" t="s">
         <v>57</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E21" s="5"/>
+        <v>47</v>
+      </c>
+      <c r="E21" s="5" t="s">
+        <v>55</v>
+      </c>
       <c r="F21" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G21" s="1" t="n">
         <v>0</v>
@@ -2532,13 +2391,13 @@
         <v>58</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C22" s="1" t="s">
         <v>59</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E22" s="5"/>
       <c r="F22" s="1" t="n">
@@ -2553,30 +2412,34 @@
         <v>60</v>
       </c>
       <c r="B23" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="C23" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="C23" s="1" t="s">
-        <v>62</v>
-      </c>
       <c r="D23" s="1" t="s">
-        <v>45</v>
-      </c>
+        <v>47</v>
+      </c>
+      <c r="E23" s="5"/>
       <c r="F23" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="B24" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="B24" s="3" t="s">
-        <v>61</v>
-      </c>
       <c r="C24" s="1" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F24" s="1" t="n">
         <v>0</v>
@@ -2584,16 +2447,16 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="C25" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="B25" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>65</v>
-      </c>
       <c r="D25" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F25" s="1" t="n">
         <v>0</v>
@@ -2604,13 +2467,13 @@
         <v>66</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F26" s="1" t="n">
         <v>0</v>
@@ -2618,16 +2481,16 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="C27" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="B27" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="C27" s="1" t="s">
-        <v>68</v>
-      </c>
       <c r="D27" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F27" s="1" t="n">
         <v>0</v>
@@ -2638,13 +2501,13 @@
         <v>69</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F28" s="1" t="n">
         <v>0</v>
@@ -2652,51 +2515,45 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="C29" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="B29" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="C29" s="1" t="s">
-        <v>71</v>
-      </c>
       <c r="D29" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E29" s="1" t="s">
-        <v>72</v>
+        <v>47</v>
       </c>
       <c r="F29" s="1" t="n">
         <v>0</v>
-      </c>
-      <c r="G29" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H29" s="1" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="C30" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="B30" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="C30" s="1" t="s">
+      <c r="D30" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E30" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="D30" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E30" s="1" t="s">
-        <v>53</v>
-      </c>
       <c r="F30" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G30" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="H30" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2704,30 +2561,36 @@
         <v>75</v>
       </c>
       <c r="B31" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="C31" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="C31" s="1" t="s">
-        <v>77</v>
-      </c>
       <c r="D31" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>55</v>
       </c>
       <c r="F31" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="B32" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="B32" s="3" t="s">
-        <v>76</v>
-      </c>
       <c r="C32" s="1" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F32" s="1" t="n">
         <v>0</v>
@@ -2735,16 +2598,16 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="C33" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="B33" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="C33" s="1" t="s">
-        <v>77</v>
-      </c>
       <c r="D33" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F33" s="1" t="n">
         <v>0</v>
@@ -2752,16 +2615,16 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="3" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F34" s="1" t="n">
         <v>0</v>
@@ -2772,13 +2635,13 @@
         <v>82</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F35" s="1" t="n">
         <v>0</v>
@@ -2786,16 +2649,16 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="B36" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="C36" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="B36" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="C36" s="1" t="s">
-        <v>81</v>
-      </c>
       <c r="D36" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F36" s="1" t="n">
         <v>0</v>
@@ -2803,16 +2666,16 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="3" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F37" s="1" t="n">
         <v>0</v>
@@ -2820,16 +2683,16 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="3" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F38" s="1" t="n">
         <v>0</v>
@@ -2837,16 +2700,16 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="3" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F39" s="1" t="n">
         <v>0</v>
@@ -2854,16 +2717,16 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="3" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F40" s="1" t="n">
         <v>0</v>
@@ -2874,13 +2737,13 @@
         <v>89</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F41" s="1" t="n">
         <v>0</v>
@@ -2888,16 +2751,16 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="B42" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="C42" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="B42" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="C42" s="1" t="s">
-        <v>91</v>
-      </c>
       <c r="D42" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F42" s="1" t="n">
         <v>0</v>
@@ -2908,13 +2771,13 @@
         <v>92</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F43" s="1" t="n">
         <v>0</v>
@@ -2922,93 +2785,90 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="B44" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="C44" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="B44" s="6" t="s">
-        <v>94</v>
-      </c>
-      <c r="C44" s="1" t="s">
-        <v>95</v>
-      </c>
       <c r="D44" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E44" s="5" t="s">
-        <v>96</v>
+        <v>47</v>
       </c>
       <c r="F44" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G44" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="B45" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="C45" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="B45" s="6" t="s">
-        <v>94</v>
-      </c>
-      <c r="C45" s="1" t="s">
+      <c r="D45" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E45" s="5" t="s">
         <v>98</v>
       </c>
-      <c r="D45" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E45" s="5" t="s">
-        <v>99</v>
-      </c>
       <c r="F45" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G45" s="1" t="n">
         <v>0</v>
-      </c>
-      <c r="H45" s="1" t="n">
-        <v>365</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="B46" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="C46" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="B46" s="6" t="s">
-        <v>94</v>
-      </c>
-      <c r="C46" s="1" t="s">
+      <c r="D46" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E46" s="5" t="s">
         <v>101</v>
       </c>
-      <c r="D46" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E46" s="5" t="s">
-        <v>102</v>
-      </c>
       <c r="F46" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G46" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="H46" s="1" t="n">
+        <v>365</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="B47" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="C47" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="B47" s="6" t="s">
-        <v>94</v>
-      </c>
-      <c r="C47" s="1" t="s">
+      <c r="D47" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E47" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="D47" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E47" s="5" t="s">
-        <v>102</v>
-      </c>
       <c r="F47" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G47" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3017,16 +2877,16 @@
         <v>105</v>
       </c>
       <c r="B48" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="C48" s="1" t="s">
         <v>106</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E48" s="5" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="F48" s="1" t="n">
         <v>0</v>
@@ -3037,16 +2897,16 @@
         <v>107</v>
       </c>
       <c r="B49" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="C49" s="1" t="s">
         <v>108</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E49" s="5" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="F49" s="1" t="n">
         <v>0</v>
@@ -3054,19 +2914,19 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="B50" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="C50" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="B50" s="6" t="s">
-        <v>94</v>
-      </c>
-      <c r="C50" s="1" t="s">
+      <c r="D50" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E50" s="5" t="s">
         <v>111</v>
-      </c>
-      <c r="D50" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E50" s="5" t="s">
-        <v>102</v>
       </c>
       <c r="F50" s="1" t="n">
         <v>0</v>
@@ -3077,42 +2937,36 @@
         <v>112</v>
       </c>
       <c r="B51" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="C51" s="1" t="s">
         <v>113</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>14</v>
+        <v>47</v>
       </c>
       <c r="E51" s="5" t="s">
-        <v>114</v>
+        <v>104</v>
       </c>
       <c r="F51" s="1" t="n">
         <v>0</v>
-      </c>
-      <c r="G51" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H51" s="1" t="n">
-        <v>2</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="B52" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="C52" s="1" t="s">
         <v>115</v>
-      </c>
-      <c r="B52" s="6" t="s">
-        <v>94</v>
-      </c>
-      <c r="C52" s="1" t="s">
-        <v>116</v>
       </c>
       <c r="D52" s="1" t="s">
         <v>14</v>
       </c>
       <c r="E52" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="F52" s="1" t="n">
         <v>0</v>
@@ -3129,39 +2983,42 @@
         <v>117</v>
       </c>
       <c r="B53" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="C53" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="C53" s="1" t="s">
-        <v>119</v>
-      </c>
       <c r="D53" s="1" t="s">
-        <v>45</v>
+        <v>14</v>
       </c>
       <c r="E53" s="5" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="F53" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G53" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="H53" s="1" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="B54" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="C54" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="B54" s="6" t="s">
-        <v>118</v>
-      </c>
-      <c r="C54" s="1" t="s">
+      <c r="D54" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E54" s="5" t="s">
         <v>122</v>
-      </c>
-      <c r="D54" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E54" s="1" t="s">
-        <v>123</v>
       </c>
       <c r="F54" s="1" t="n">
         <v>0</v>
@@ -3172,19 +3029,19 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="B55" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="C55" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="B55" s="6" t="s">
-        <v>118</v>
-      </c>
-      <c r="C55" s="1" t="s">
+      <c r="D55" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E55" s="1" t="s">
         <v>125</v>
-      </c>
-      <c r="D55" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E55" s="1" t="s">
-        <v>123</v>
       </c>
       <c r="F55" s="1" t="n">
         <v>0</v>
@@ -3198,16 +3055,16 @@
         <v>126</v>
       </c>
       <c r="B56" s="6" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C56" s="1" t="s">
         <v>127</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E56" s="1" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="F56" s="1" t="n">
         <v>0</v>
@@ -3221,73 +3078,70 @@
         <v>128</v>
       </c>
       <c r="B57" s="6" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C57" s="1" t="s">
         <v>129</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E57" s="1" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="F57" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G57" s="1" t="n">
         <v>0</v>
-      </c>
-      <c r="H57" s="1" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="B58" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="C58" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="B58" s="6" t="s">
-        <v>118</v>
-      </c>
-      <c r="C58" s="1" t="s">
+      <c r="D58" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E58" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="D58" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E58" s="5" t="s">
-        <v>133</v>
-      </c>
       <c r="F58" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G58" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H58" s="1" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="B59" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="C59" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="B59" s="6" t="s">
-        <v>118</v>
-      </c>
-      <c r="C59" s="1" t="s">
+      <c r="D59" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E59" s="5" t="s">
         <v>135</v>
       </c>
-      <c r="D59" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E59" s="5" t="s">
-        <v>130</v>
-      </c>
       <c r="F59" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G59" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H59" s="1" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3296,39 +3150,42 @@
         <v>136</v>
       </c>
       <c r="B60" s="6" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C60" s="1" t="s">
         <v>137</v>
       </c>
       <c r="D60" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E60" s="1" t="s">
-        <v>138</v>
+        <v>47</v>
+      </c>
+      <c r="E60" s="5" t="s">
+        <v>132</v>
       </c>
       <c r="F60" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G60" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="H60" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="B61" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="C61" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="B61" s="6" t="s">
-        <v>118</v>
-      </c>
-      <c r="C61" s="1" t="s">
+      <c r="D61" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E61" s="1" t="s">
         <v>140</v>
-      </c>
-      <c r="D61" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E61" s="7" t="s">
-        <v>138</v>
       </c>
       <c r="F61" s="1" t="n">
         <v>0</v>
@@ -3342,16 +3199,16 @@
         <v>141</v>
       </c>
       <c r="B62" s="6" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C62" s="1" t="s">
         <v>142</v>
       </c>
       <c r="D62" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E62" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
+      </c>
+      <c r="E62" s="7" t="s">
+        <v>140</v>
       </c>
       <c r="F62" s="1" t="n">
         <v>0</v>
@@ -3365,16 +3222,16 @@
         <v>143</v>
       </c>
       <c r="B63" s="6" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C63" s="1" t="s">
         <v>144</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E63" s="1" t="s">
-        <v>145</v>
+        <v>48</v>
       </c>
       <c r="F63" s="1" t="n">
         <v>0</v>
@@ -3385,19 +3242,19 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="B64" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="C64" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="B64" s="6" t="s">
-        <v>118</v>
-      </c>
-      <c r="C64" s="1" t="s">
+      <c r="D64" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E64" s="1" t="s">
         <v>147</v>
-      </c>
-      <c r="D64" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E64" s="1" t="s">
-        <v>148</v>
       </c>
       <c r="F64" s="1" t="n">
         <v>0</v>
@@ -3408,19 +3265,19 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="B65" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="C65" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="B65" s="6" t="s">
+      <c r="D65" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E65" s="1" t="s">
         <v>150</v>
-      </c>
-      <c r="C65" s="1" t="s">
-        <v>151</v>
-      </c>
-      <c r="D65" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E65" s="5" t="s">
-        <v>152</v>
       </c>
       <c r="F65" s="1" t="n">
         <v>0</v>
@@ -3431,19 +3288,19 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="B66" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="C66" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="B66" s="6" t="s">
-        <v>150</v>
-      </c>
-      <c r="C66" s="1" t="s">
+      <c r="D66" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E66" s="5" t="s">
         <v>154</v>
-      </c>
-      <c r="D66" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E66" s="5" t="s">
-        <v>152</v>
       </c>
       <c r="F66" s="1" t="n">
         <v>0</v>
@@ -3457,39 +3314,39 @@
         <v>155</v>
       </c>
       <c r="B67" s="6" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="C67" s="1" t="s">
         <v>156</v>
       </c>
       <c r="D67" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E67" s="5" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="F67" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="H67" s="1" t="n">
+      <c r="G67" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="B68" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="C68" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="B68" s="6" t="s">
-        <v>150</v>
-      </c>
-      <c r="C68" s="1" t="s">
+      <c r="D68" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E68" s="5" t="s">
         <v>159</v>
-      </c>
-      <c r="D68" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E68" s="5" t="s">
-        <v>157</v>
       </c>
       <c r="F68" s="1" t="n">
         <v>0</v>
@@ -3503,21 +3360,21 @@
         <v>160</v>
       </c>
       <c r="B69" s="6" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="C69" s="1" t="s">
         <v>161</v>
       </c>
       <c r="D69" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E69" s="5" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="F69" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="G69" s="1" t="n">
+      <c r="H69" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3526,25 +3383,22 @@
         <v>162</v>
       </c>
       <c r="B70" s="6" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="C70" s="1" t="s">
         <v>163</v>
       </c>
       <c r="D70" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E70" s="5" t="s">
-        <v>130</v>
+        <v>159</v>
       </c>
       <c r="F70" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G70" s="1" t="n">
         <v>0</v>
-      </c>
-      <c r="H70" s="1" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3552,22 +3406,25 @@
         <v>164</v>
       </c>
       <c r="B71" s="6" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="C71" s="1" t="s">
         <v>165</v>
       </c>
       <c r="D71" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E71" s="5" t="s">
-        <v>157</v>
+        <v>132</v>
       </c>
       <c r="F71" s="1" t="n">
         <v>0</v>
       </c>
+      <c r="G71" s="1" t="n">
+        <v>0</v>
+      </c>
       <c r="H71" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3575,21 +3432,21 @@
         <v>166</v>
       </c>
       <c r="B72" s="6" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="C72" s="1" t="s">
         <v>167</v>
       </c>
       <c r="D72" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E72" s="5" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="F72" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="G72" s="1" t="n">
+      <c r="H72" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3598,25 +3455,22 @@
         <v>168</v>
       </c>
       <c r="B73" s="6" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="C73" s="1" t="s">
         <v>169</v>
       </c>
       <c r="D73" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E73" s="5" t="s">
-        <v>130</v>
+        <v>159</v>
       </c>
       <c r="F73" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G73" s="1" t="n">
         <v>0</v>
-      </c>
-      <c r="H73" s="1" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3624,39 +3478,42 @@
         <v>170</v>
       </c>
       <c r="B74" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="C74" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="C74" s="1" t="s">
-        <v>172</v>
-      </c>
       <c r="D74" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E74" s="5" t="s">
-        <v>173</v>
+        <v>132</v>
       </c>
       <c r="F74" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G74" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="H74" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="B75" s="6" t="s">
+        <v>173</v>
+      </c>
+      <c r="C75" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="B75" s="6" t="s">
-        <v>171</v>
-      </c>
-      <c r="C75" s="1" t="s">
+      <c r="D75" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E75" s="5" t="s">
         <v>175</v>
-      </c>
-      <c r="D75" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E75" s="5" t="s">
-        <v>176</v>
       </c>
       <c r="F75" s="1" t="n">
         <v>0</v>
@@ -3667,19 +3524,19 @@
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="B76" s="6" t="s">
+        <v>173</v>
+      </c>
+      <c r="C76" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="B76" s="6" t="s">
-        <v>171</v>
-      </c>
-      <c r="C76" s="1" t="s">
+      <c r="D76" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E76" s="5" t="s">
         <v>178</v>
-      </c>
-      <c r="D76" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E76" s="5" t="s">
-        <v>152</v>
       </c>
       <c r="F76" s="1" t="n">
         <v>0</v>
@@ -3693,16 +3550,16 @@
         <v>179</v>
       </c>
       <c r="B77" s="6" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="C77" s="1" t="s">
         <v>180</v>
       </c>
       <c r="D77" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E77" s="5" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="F77" s="1" t="n">
         <v>0</v>
@@ -3716,16 +3573,16 @@
         <v>181</v>
       </c>
       <c r="B78" s="6" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="C78" s="1" t="s">
         <v>182</v>
       </c>
       <c r="D78" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E78" s="5" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="F78" s="1" t="n">
         <v>0</v>
@@ -3739,48 +3596,48 @@
         <v>183</v>
       </c>
       <c r="B79" s="6" t="s">
+        <v>173</v>
+      </c>
+      <c r="C79" s="1" t="s">
         <v>184</v>
       </c>
-      <c r="C79" s="1" t="s">
-        <v>185</v>
-      </c>
       <c r="D79" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E79" s="5" t="s">
-        <v>186</v>
+        <v>154</v>
       </c>
       <c r="F79" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G79" s="1" t="n">
         <v>0</v>
-      </c>
-      <c r="H79" s="1" t="n">
-        <v>90</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="B80" s="6" t="s">
+        <v>186</v>
+      </c>
+      <c r="C80" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="B80" s="6" t="s">
-        <v>184</v>
-      </c>
-      <c r="C80" s="1" t="s">
+      <c r="D80" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E80" s="5" t="s">
         <v>188</v>
       </c>
-      <c r="D80" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E80" s="5" t="s">
-        <v>186</v>
-      </c>
       <c r="F80" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G80" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="H80" s="1" t="n">
+        <v>90</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3788,16 +3645,16 @@
         <v>189</v>
       </c>
       <c r="B81" s="6" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="C81" s="1" t="s">
         <v>190</v>
       </c>
       <c r="D81" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E81" s="5" t="s">
-        <v>72</v>
+        <v>188</v>
       </c>
       <c r="F81" s="1" t="n">
         <v>0</v>
@@ -3811,16 +3668,16 @@
         <v>191</v>
       </c>
       <c r="B82" s="6" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="C82" s="1" t="s">
         <v>192</v>
       </c>
       <c r="D82" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E82" s="5" t="s">
-        <v>193</v>
+        <v>74</v>
       </c>
       <c r="F82" s="1" t="n">
         <v>0</v>
@@ -3831,19 +3688,19 @@
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="B83" s="6" t="s">
+        <v>186</v>
+      </c>
+      <c r="C83" s="1" t="s">
         <v>194</v>
       </c>
-      <c r="B83" s="6" t="s">
-        <v>184</v>
-      </c>
-      <c r="C83" s="1" t="s">
+      <c r="D83" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E83" s="5" t="s">
         <v>195</v>
-      </c>
-      <c r="D83" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E83" s="5" t="s">
-        <v>193</v>
       </c>
       <c r="F83" s="1" t="n">
         <v>0</v>
@@ -3857,16 +3714,16 @@
         <v>196</v>
       </c>
       <c r="B84" s="6" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="C84" s="1" t="s">
         <v>197</v>
       </c>
       <c r="D84" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E84" s="5" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="F84" s="1" t="n">
         <v>0</v>
@@ -3880,16 +3737,16 @@
         <v>198</v>
       </c>
       <c r="B85" s="6" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="C85" s="1" t="s">
         <v>199</v>
       </c>
       <c r="D85" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E85" s="5" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="F85" s="1" t="n">
         <v>0</v>
@@ -3900,34 +3757,39 @@
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="3" t="s">
+        <v>200</v>
+      </c>
+      <c r="B86" s="6" t="s">
+        <v>186</v>
+      </c>
+      <c r="C86" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="B86" s="6" t="s">
+      <c r="D86" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E86" s="5" t="s">
         <v>202</v>
       </c>
-      <c r="C86" s="1" t="s">
-        <v>203</v>
-      </c>
-      <c r="D86" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E86" s="5"/>
       <c r="F86" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G86" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="3" t="s">
+        <v>203</v>
+      </c>
+      <c r="B87" s="6" t="s">
         <v>204</v>
-      </c>
-      <c r="B87" s="6" t="s">
-        <v>202</v>
       </c>
       <c r="C87" s="1" t="s">
         <v>205</v>
       </c>
       <c r="D87" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E87" s="5"/>
       <c r="F87" s="1" t="n">
@@ -3939,42 +3801,39 @@
         <v>206</v>
       </c>
       <c r="B88" s="6" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="C88" s="1" t="s">
         <v>207</v>
       </c>
       <c r="D88" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E88" s="5" t="s">
-        <v>208</v>
-      </c>
+        <v>47</v>
+      </c>
+      <c r="E88" s="5"/>
       <c r="F88" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H88" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="3" t="s">
+        <v>208</v>
+      </c>
+      <c r="B89" s="6" t="s">
+        <v>204</v>
+      </c>
+      <c r="C89" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="B89" s="6" t="s">
-        <v>202</v>
-      </c>
-      <c r="C89" s="1" t="s">
+      <c r="D89" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E89" s="5" t="s">
         <v>210</v>
       </c>
-      <c r="D89" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E89" s="5"/>
       <c r="F89" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="G89" s="1" t="n">
+      <c r="H89" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3983,17 +3842,15 @@
         <v>211</v>
       </c>
       <c r="B90" s="6" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="C90" s="1" t="s">
         <v>212</v>
       </c>
       <c r="D90" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E90" s="5" t="s">
-        <v>213</v>
-      </c>
+        <v>47</v>
+      </c>
+      <c r="E90" s="5"/>
       <c r="F90" s="1" t="n">
         <v>0</v>
       </c>
@@ -4003,19 +3860,24 @@
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="B91" s="6" t="s">
+        <v>204</v>
+      </c>
+      <c r="C91" s="1" t="s">
         <v>214</v>
       </c>
-      <c r="B91" s="6" t="s">
-        <v>202</v>
-      </c>
-      <c r="C91" s="1" t="s">
+      <c r="D91" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E91" s="5" t="s">
         <v>215</v>
       </c>
-      <c r="D91" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E91" s="5"/>
       <c r="F91" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G91" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4024,13 +3886,13 @@
         <v>216</v>
       </c>
       <c r="B92" s="6" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="C92" s="1" t="s">
         <v>217</v>
       </c>
       <c r="D92" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E92" s="5"/>
       <c r="F92" s="1" t="n">
@@ -4042,57 +3904,52 @@
         <v>218</v>
       </c>
       <c r="B93" s="6" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="C93" s="1" t="s">
         <v>219</v>
       </c>
       <c r="D93" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E93" s="5"/>
       <c r="F93" s="1" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="94" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="3" t="s">
         <v>220</v>
       </c>
       <c r="B94" s="6" t="s">
-        <v>202</v>
-      </c>
-      <c r="C94" s="8" t="s">
+        <v>204</v>
+      </c>
+      <c r="C94" s="1" t="s">
         <v>221</v>
       </c>
       <c r="D94" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E94" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="E94" s="5"/>
+      <c r="F94" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="95" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A95" s="3" t="s">
         <v>222</v>
       </c>
-      <c r="F94" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G94" s="1" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A95" s="3" t="s">
+      <c r="B95" s="6" t="s">
+        <v>204</v>
+      </c>
+      <c r="C95" s="8" t="s">
         <v>223</v>
       </c>
-      <c r="B95" s="6" t="s">
-        <v>202</v>
-      </c>
-      <c r="C95" s="1" t="s">
+      <c r="D95" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E95" s="5" t="s">
         <v>224</v>
-      </c>
-      <c r="D95" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E95" s="5" t="s">
-        <v>222</v>
       </c>
       <c r="F95" s="1" t="n">
         <v>0</v>
@@ -4106,35 +3963,40 @@
         <v>225</v>
       </c>
       <c r="B96" s="6" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="C96" s="1" t="s">
         <v>226</v>
       </c>
       <c r="D96" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E96" s="5" t="s">
-        <v>102</v>
+        <v>224</v>
       </c>
       <c r="F96" s="1" t="n">
         <v>0</v>
       </c>
-    </row>
-    <row r="97" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G96" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="3" t="s">
         <v>227</v>
       </c>
       <c r="B97" s="6" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="C97" s="1" t="s">
         <v>228</v>
       </c>
       <c r="D97" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E97" s="5"/>
+        <v>47</v>
+      </c>
+      <c r="E97" s="5" t="s">
+        <v>104</v>
+      </c>
       <c r="F97" s="1" t="n">
         <v>0</v>
       </c>
@@ -4144,44 +4006,39 @@
         <v>229</v>
       </c>
       <c r="B98" s="6" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="C98" s="1" t="s">
         <v>230</v>
       </c>
       <c r="D98" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E98" s="5" t="s">
-        <v>231</v>
-      </c>
+        <v>47</v>
+      </c>
+      <c r="E98" s="5"/>
       <c r="F98" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G98" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="3" t="s">
+        <v>231</v>
+      </c>
+      <c r="B99" s="6" t="s">
+        <v>204</v>
+      </c>
+      <c r="C99" s="1" t="s">
         <v>232</v>
       </c>
-      <c r="B99" s="6" t="s">
-        <v>202</v>
-      </c>
-      <c r="C99" s="1" t="s">
+      <c r="D99" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E99" s="5" t="s">
         <v>233</v>
       </c>
-      <c r="D99" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E99" s="5" t="s">
-        <v>208</v>
-      </c>
       <c r="F99" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="H99" s="1" t="n">
+      <c r="G99" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4190,86 +4047,86 @@
         <v>234</v>
       </c>
       <c r="B100" s="6" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="C100" s="1" t="s">
         <v>235</v>
       </c>
       <c r="D100" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E100" s="5" t="s">
+        <v>210</v>
+      </c>
+      <c r="F100" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H100" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="101" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A101" s="3" t="s">
         <v>236</v>
       </c>
-      <c r="F100" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G100" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H100" s="1"/>
-    </row>
-    <row r="101" customFormat="false" ht="16.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A101" s="3" t="s">
+      <c r="B101" s="6" t="s">
+        <v>204</v>
+      </c>
+      <c r="C101" s="1" t="s">
         <v>237</v>
       </c>
-      <c r="B101" s="6" t="s">
-        <v>202</v>
-      </c>
-      <c r="C101" s="1" t="s">
+      <c r="D101" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E101" s="5" t="s">
         <v>238</v>
       </c>
-      <c r="D101" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E101" s="5" t="s">
+      <c r="F101" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G101" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H101" s="1"/>
+    </row>
+    <row r="102" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A102" s="3" t="s">
         <v>239</v>
       </c>
-      <c r="F101" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G101" s="1" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A102" s="3" t="s">
+      <c r="B102" s="6" t="s">
+        <v>204</v>
+      </c>
+      <c r="C102" s="1" t="s">
         <v>240</v>
       </c>
-      <c r="B102" s="6" t="s">
-        <v>202</v>
-      </c>
-      <c r="C102" s="1" t="s">
+      <c r="D102" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E102" s="5" t="s">
         <v>241</v>
       </c>
-      <c r="D102" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E102" s="5" t="s">
-        <v>208</v>
-      </c>
       <c r="F102" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="H102" s="1" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="103" customFormat="false" ht="16.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G102" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="3" t="s">
         <v>242</v>
       </c>
       <c r="B103" s="6" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="C103" s="1" t="s">
         <v>243</v>
       </c>
       <c r="D103" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E103" s="5" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="F103" s="1" t="n">
         <v>0</v>
@@ -4278,21 +4135,21 @@
         <v>0</v>
       </c>
     </row>
-    <row r="104" customFormat="false" ht="16.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="104" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="3" t="s">
         <v>244</v>
       </c>
       <c r="B104" s="6" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="C104" s="1" t="s">
         <v>245</v>
       </c>
       <c r="D104" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E104" s="5" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="F104" s="1" t="n">
         <v>0</v>
@@ -4301,68 +4158,68 @@
         <v>0</v>
       </c>
     </row>
-    <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="105" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="3" t="s">
         <v>246</v>
       </c>
       <c r="B105" s="6" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="C105" s="1" t="s">
         <v>247</v>
       </c>
       <c r="D105" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E105" s="5" t="s">
-        <v>236</v>
+        <v>210</v>
       </c>
       <c r="F105" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="G105" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H105" s="1"/>
+      <c r="H105" s="1" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="3" t="s">
         <v>248</v>
       </c>
       <c r="B106" s="6" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="C106" s="1" t="s">
         <v>249</v>
       </c>
       <c r="D106" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E106" s="5" t="s">
-        <v>208</v>
+        <v>238</v>
       </c>
       <c r="F106" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="H106" s="1" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="107" customFormat="false" ht="16.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G106" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H106" s="1"/>
+    </row>
+    <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="3" t="s">
         <v>250</v>
       </c>
       <c r="B107" s="6" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="C107" s="1" t="s">
         <v>251</v>
       </c>
       <c r="D107" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E107" s="5" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="F107" s="1" t="n">
         <v>0</v>
@@ -4371,21 +4228,21 @@
         <v>0</v>
       </c>
     </row>
-    <row r="108" customFormat="false" ht="16.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="108" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="3" t="s">
         <v>252</v>
       </c>
       <c r="B108" s="6" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="C108" s="1" t="s">
         <v>253</v>
       </c>
       <c r="D108" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E108" s="5" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="F108" s="1" t="n">
         <v>0</v>
@@ -4394,45 +4251,44 @@
         <v>0</v>
       </c>
     </row>
-    <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="109" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="3" t="s">
         <v>254</v>
       </c>
       <c r="B109" s="6" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="C109" s="1" t="s">
         <v>255</v>
       </c>
       <c r="D109" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E109" s="5" t="s">
-        <v>236</v>
+        <v>210</v>
       </c>
       <c r="F109" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="G109" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H109" s="1"/>
+      <c r="H109" s="1" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="3" t="s">
         <v>256</v>
       </c>
       <c r="B110" s="6" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="C110" s="1" t="s">
         <v>257</v>
       </c>
       <c r="D110" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E110" s="5" t="s">
-        <v>258</v>
+        <v>238</v>
       </c>
       <c r="F110" s="1" t="n">
         <v>0</v>
@@ -4440,27 +4296,28 @@
       <c r="G110" s="1" t="n">
         <v>0</v>
       </c>
+      <c r="H110" s="1"/>
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A111" s="3" t="s">
+        <v>258</v>
+      </c>
+      <c r="B111" s="6" t="s">
+        <v>204</v>
+      </c>
+      <c r="C111" s="1" t="s">
         <v>259</v>
       </c>
-      <c r="B111" s="6" t="s">
-        <v>202</v>
-      </c>
-      <c r="C111" s="1" t="s">
+      <c r="D111" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E111" s="5" t="s">
         <v>260</v>
       </c>
-      <c r="D111" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E111" s="5" t="s">
-        <v>208</v>
-      </c>
       <c r="F111" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="H111" s="1" t="n">
+      <c r="G111" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4469,16 +4326,16 @@
         <v>261</v>
       </c>
       <c r="B112" s="6" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="C112" s="1" t="s">
         <v>262</v>
       </c>
       <c r="D112" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E112" s="5" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="F112" s="1" t="n">
         <v>0</v>
@@ -4492,16 +4349,16 @@
         <v>263</v>
       </c>
       <c r="B113" s="6" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="C113" s="1" t="s">
         <v>264</v>
       </c>
       <c r="D113" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E113" s="5" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="F113" s="1" t="n">
         <v>0</v>
@@ -4515,40 +4372,39 @@
         <v>265</v>
       </c>
       <c r="B114" s="6" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="C114" s="1" t="s">
         <v>266</v>
       </c>
       <c r="D114" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E114" s="5" t="s">
-        <v>236</v>
+        <v>210</v>
       </c>
       <c r="F114" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="G114" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H114" s="1"/>
+      <c r="H114" s="1" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A115" s="3" t="s">
         <v>267</v>
       </c>
       <c r="B115" s="6" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="C115" s="1" t="s">
         <v>268</v>
       </c>
       <c r="D115" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E115" s="5" t="s">
-        <v>258</v>
+        <v>238</v>
       </c>
       <c r="F115" s="1" t="n">
         <v>0</v>
@@ -4556,27 +4412,28 @@
       <c r="G115" s="1" t="n">
         <v>0</v>
       </c>
+      <c r="H115" s="1"/>
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A116" s="3" t="s">
         <v>269</v>
       </c>
       <c r="B116" s="6" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="C116" s="1" t="s">
         <v>270</v>
       </c>
       <c r="D116" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E116" s="5" t="s">
-        <v>208</v>
+        <v>260</v>
       </c>
       <c r="F116" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="H116" s="1" t="n">
+      <c r="G116" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4585,16 +4442,16 @@
         <v>271</v>
       </c>
       <c r="B117" s="6" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="C117" s="1" t="s">
         <v>272</v>
       </c>
       <c r="D117" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E117" s="5" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="F117" s="1" t="n">
         <v>0</v>
@@ -4608,16 +4465,16 @@
         <v>273</v>
       </c>
       <c r="B118" s="6" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="C118" s="1" t="s">
         <v>274</v>
       </c>
       <c r="D118" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E118" s="5" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="F118" s="1" t="n">
         <v>0</v>
@@ -4631,40 +4488,39 @@
         <v>275</v>
       </c>
       <c r="B119" s="6" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="C119" s="1" t="s">
         <v>276</v>
       </c>
       <c r="D119" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E119" s="5" t="s">
-        <v>236</v>
+        <v>210</v>
       </c>
       <c r="F119" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="G119" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H119" s="1"/>
+      <c r="H119" s="1" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A120" s="3" t="s">
         <v>277</v>
       </c>
       <c r="B120" s="6" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="C120" s="1" t="s">
         <v>278</v>
       </c>
       <c r="D120" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E120" s="9" t="s">
-        <v>279</v>
+        <v>47</v>
+      </c>
+      <c r="E120" s="5" t="s">
+        <v>238</v>
       </c>
       <c r="F120" s="1" t="n">
         <v>0</v>
@@ -4672,22 +4528,23 @@
       <c r="G120" s="1" t="n">
         <v>0</v>
       </c>
+      <c r="H120" s="1"/>
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A121" s="3" t="s">
+        <v>279</v>
+      </c>
+      <c r="B121" s="6" t="s">
+        <v>204</v>
+      </c>
+      <c r="C121" s="1" t="s">
         <v>280</v>
       </c>
-      <c r="B121" s="6" t="s">
-        <v>202</v>
-      </c>
-      <c r="C121" s="1" t="s">
+      <c r="D121" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E121" s="9" t="s">
         <v>281</v>
-      </c>
-      <c r="D121" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E121" s="9" t="s">
-        <v>282</v>
       </c>
       <c r="F121" s="1" t="n">
         <v>0</v>
@@ -4698,19 +4555,19 @@
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A122" s="3" t="s">
+        <v>282</v>
+      </c>
+      <c r="B122" s="6" t="s">
+        <v>204</v>
+      </c>
+      <c r="C122" s="1" t="s">
         <v>283</v>
       </c>
-      <c r="B122" s="6" t="s">
-        <v>202</v>
-      </c>
-      <c r="C122" s="1" t="s">
+      <c r="D122" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E122" s="9" t="s">
         <v>284</v>
-      </c>
-      <c r="D122" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E122" s="1" t="s">
-        <v>285</v>
       </c>
       <c r="F122" s="1" t="n">
         <v>0</v>
@@ -4721,19 +4578,19 @@
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A123" s="3" t="s">
+        <v>285</v>
+      </c>
+      <c r="B123" s="6" t="s">
+        <v>204</v>
+      </c>
+      <c r="C123" s="1" t="s">
         <v>286</v>
       </c>
-      <c r="B123" s="3" t="s">
+      <c r="D123" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E123" s="1" t="s">
         <v>287</v>
-      </c>
-      <c r="C123" s="1" t="s">
-        <v>288</v>
-      </c>
-      <c r="D123" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E123" s="1" t="s">
-        <v>285</v>
       </c>
       <c r="F123" s="1" t="n">
         <v>0</v>
@@ -4744,19 +4601,19 @@
     </row>
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A124" s="3" t="s">
+        <v>288</v>
+      </c>
+      <c r="B124" s="3" t="s">
         <v>289</v>
-      </c>
-      <c r="B124" s="3" t="s">
-        <v>287</v>
       </c>
       <c r="C124" s="1" t="s">
         <v>290</v>
       </c>
       <c r="D124" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E124" s="1" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="F124" s="1" t="n">
         <v>0</v>
@@ -4770,16 +4627,16 @@
         <v>291</v>
       </c>
       <c r="B125" s="3" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="C125" s="1" t="s">
         <v>292</v>
       </c>
       <c r="D125" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E125" s="1" t="s">
-        <v>293</v>
+        <v>287</v>
       </c>
       <c r="F125" s="1" t="n">
         <v>0</v>
@@ -4790,19 +4647,19 @@
     </row>
     <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A126" s="3" t="s">
+        <v>293</v>
+      </c>
+      <c r="B126" s="3" t="s">
+        <v>289</v>
+      </c>
+      <c r="C126" s="1" t="s">
         <v>294</v>
       </c>
-      <c r="B126" s="3" t="s">
-        <v>287</v>
-      </c>
-      <c r="C126" s="1" t="s">
+      <c r="D126" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E126" s="1" t="s">
         <v>295</v>
-      </c>
-      <c r="D126" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E126" s="7" t="s">
-        <v>296</v>
       </c>
       <c r="F126" s="1" t="n">
         <v>0</v>
@@ -4813,19 +4670,19 @@
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A127" s="3" t="s">
+        <v>296</v>
+      </c>
+      <c r="B127" s="3" t="s">
+        <v>289</v>
+      </c>
+      <c r="C127" s="1" t="s">
         <v>297</v>
       </c>
-      <c r="B127" s="3" t="s">
-        <v>287</v>
-      </c>
-      <c r="C127" s="1" t="s">
+      <c r="D127" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E127" s="7" t="s">
         <v>298</v>
-      </c>
-      <c r="D127" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E127" s="7" t="s">
-        <v>296</v>
       </c>
       <c r="F127" s="1" t="n">
         <v>0</v>
@@ -4839,16 +4696,16 @@
         <v>299</v>
       </c>
       <c r="B128" s="3" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="C128" s="1" t="s">
         <v>300</v>
       </c>
       <c r="D128" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E128" s="7" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="F128" s="1" t="n">
         <v>0</v>
@@ -4862,16 +4719,16 @@
         <v>301</v>
       </c>
       <c r="B129" s="3" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="C129" s="1" t="s">
         <v>302</v>
       </c>
       <c r="D129" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E129" s="7" t="s">
-        <v>303</v>
+        <v>298</v>
       </c>
       <c r="F129" s="1" t="n">
         <v>0</v>
@@ -4882,19 +4739,19 @@
     </row>
     <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A130" s="3" t="s">
+        <v>303</v>
+      </c>
+      <c r="B130" s="3" t="s">
+        <v>289</v>
+      </c>
+      <c r="C130" s="1" t="s">
         <v>304</v>
       </c>
-      <c r="B130" s="3" t="s">
-        <v>287</v>
-      </c>
-      <c r="C130" s="1" t="s">
+      <c r="D130" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E130" s="7" t="s">
         <v>305</v>
-      </c>
-      <c r="D130" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E130" s="7" t="s">
-        <v>303</v>
       </c>
       <c r="F130" s="1" t="n">
         <v>0</v>
@@ -4908,16 +4765,16 @@
         <v>306</v>
       </c>
       <c r="B131" s="3" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="C131" s="1" t="s">
         <v>307</v>
       </c>
       <c r="D131" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E131" s="7" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="F131" s="1" t="n">
         <v>0</v>
@@ -4931,16 +4788,16 @@
         <v>308</v>
       </c>
       <c r="B132" s="3" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="C132" s="1" t="s">
         <v>309</v>
       </c>
       <c r="D132" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E132" s="7" t="s">
-        <v>310</v>
+        <v>305</v>
       </c>
       <c r="F132" s="1" t="n">
         <v>0</v>
@@ -4951,19 +4808,19 @@
     </row>
     <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A133" s="3" t="s">
+        <v>310</v>
+      </c>
+      <c r="B133" s="3" t="s">
+        <v>289</v>
+      </c>
+      <c r="C133" s="1" t="s">
         <v>311</v>
       </c>
-      <c r="B133" s="3" t="s">
-        <v>287</v>
-      </c>
-      <c r="C133" s="1" t="s">
+      <c r="D133" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E133" s="7" t="s">
         <v>312</v>
-      </c>
-      <c r="D133" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E133" s="1" t="s">
-        <v>313</v>
       </c>
       <c r="F133" s="1" t="n">
         <v>0</v>
@@ -4974,19 +4831,19 @@
     </row>
     <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A134" s="3" t="s">
+        <v>313</v>
+      </c>
+      <c r="B134" s="3" t="s">
+        <v>289</v>
+      </c>
+      <c r="C134" s="1" t="s">
         <v>314</v>
       </c>
-      <c r="B134" s="3" t="s">
-        <v>287</v>
-      </c>
-      <c r="C134" s="1" t="s">
+      <c r="D134" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E134" s="1" t="s">
         <v>315</v>
-      </c>
-      <c r="D134" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E134" s="1" t="s">
-        <v>316</v>
       </c>
       <c r="F134" s="1" t="n">
         <v>0</v>
@@ -4997,19 +4854,19 @@
     </row>
     <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A135" s="3" t="s">
+        <v>316</v>
+      </c>
+      <c r="B135" s="3" t="s">
+        <v>289</v>
+      </c>
+      <c r="C135" s="1" t="s">
         <v>317</v>
       </c>
-      <c r="B135" s="3" t="s">
-        <v>287</v>
-      </c>
-      <c r="C135" s="1" t="s">
+      <c r="D135" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E135" s="1" t="s">
         <v>318</v>
-      </c>
-      <c r="D135" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E135" s="1" t="s">
-        <v>319</v>
       </c>
       <c r="F135" s="1" t="n">
         <v>0</v>
@@ -5020,19 +4877,19 @@
     </row>
     <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A136" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="B136" s="3" t="s">
+        <v>289</v>
+      </c>
+      <c r="C136" s="1" t="s">
         <v>320</v>
       </c>
-      <c r="B136" s="3" t="s">
-        <v>287</v>
-      </c>
-      <c r="C136" s="1" t="s">
+      <c r="D136" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E136" s="1" t="s">
         <v>321</v>
-      </c>
-      <c r="D136" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E136" s="1" t="s">
-        <v>322</v>
       </c>
       <c r="F136" s="1" t="n">
         <v>0</v>
@@ -5043,19 +4900,19 @@
     </row>
     <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A137" s="3" t="s">
+        <v>322</v>
+      </c>
+      <c r="B137" s="3" t="s">
+        <v>289</v>
+      </c>
+      <c r="C137" s="1" t="s">
         <v>323</v>
       </c>
-      <c r="B137" s="3" t="s">
-        <v>287</v>
-      </c>
-      <c r="C137" s="1" t="s">
+      <c r="D137" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E137" s="1" t="s">
         <v>324</v>
-      </c>
-      <c r="D137" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E137" s="1" t="s">
-        <v>325</v>
       </c>
       <c r="F137" s="1" t="n">
         <v>0</v>
@@ -5066,19 +4923,19 @@
     </row>
     <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A138" s="3" t="s">
+        <v>325</v>
+      </c>
+      <c r="B138" s="3" t="s">
+        <v>289</v>
+      </c>
+      <c r="C138" s="1" t="s">
         <v>326</v>
       </c>
-      <c r="B138" s="3" t="s">
-        <v>287</v>
-      </c>
-      <c r="C138" s="1" t="s">
+      <c r="D138" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E138" s="1" t="s">
         <v>327</v>
-      </c>
-      <c r="D138" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E138" s="1" t="s">
-        <v>325</v>
       </c>
       <c r="F138" s="1" t="n">
         <v>0</v>
@@ -5092,25 +4949,22 @@
         <v>328</v>
       </c>
       <c r="B139" s="3" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="C139" s="1" t="s">
         <v>329</v>
       </c>
       <c r="D139" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E139" s="1" t="s">
-        <v>72</v>
+        <v>327</v>
       </c>
       <c r="F139" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G139" s="1" t="n">
         <v>0</v>
-      </c>
-      <c r="H139" s="1" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5118,39 +4972,42 @@
         <v>330</v>
       </c>
       <c r="B140" s="3" t="s">
+        <v>289</v>
+      </c>
+      <c r="C140" s="1" t="s">
         <v>331</v>
       </c>
-      <c r="C140" s="1" t="s">
-        <v>332</v>
-      </c>
       <c r="D140" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E140" s="1" t="s">
-        <v>333</v>
+        <v>74</v>
       </c>
       <c r="F140" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G140" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="H140" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A141" s="3" t="s">
+        <v>332</v>
+      </c>
+      <c r="B141" s="3" t="s">
+        <v>333</v>
+      </c>
+      <c r="C141" s="1" t="s">
         <v>334</v>
       </c>
-      <c r="B141" s="3" t="s">
-        <v>331</v>
-      </c>
-      <c r="C141" s="1" t="s">
+      <c r="D141" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E141" s="1" t="s">
         <v>335</v>
-      </c>
-      <c r="D141" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E141" s="1" t="s">
-        <v>336</v>
       </c>
       <c r="F141" s="1" t="n">
         <v>0</v>
@@ -5161,18 +5018,24 @@
     </row>
     <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A142" s="3" t="s">
+        <v>336</v>
+      </c>
+      <c r="B142" s="3" t="s">
+        <v>333</v>
+      </c>
+      <c r="C142" s="1" t="s">
         <v>337</v>
       </c>
-      <c r="B142" s="3" t="s">
-        <v>331</v>
-      </c>
-      <c r="C142" s="1" t="s">
+      <c r="D142" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E142" s="1" t="s">
         <v>338</v>
       </c>
-      <c r="D142" s="1" t="s">
-        <v>45</v>
-      </c>
       <c r="F142" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G142" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5181,56 +5044,50 @@
         <v>339</v>
       </c>
       <c r="B143" s="3" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="C143" s="1" t="s">
         <v>340</v>
       </c>
       <c r="D143" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F143" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A144" s="7" t="s">
+      <c r="A144" s="3" t="s">
         <v>341</v>
       </c>
-      <c r="B144" s="7" t="s">
+      <c r="B144" s="3" t="s">
+        <v>333</v>
+      </c>
+      <c r="C144" s="1" t="s">
         <v>342</v>
       </c>
-      <c r="C144" s="1" t="s">
-        <v>343</v>
-      </c>
       <c r="D144" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E144" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F144" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G144" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A145" s="7" t="s">
+        <v>343</v>
+      </c>
+      <c r="B145" s="7" t="s">
         <v>344</v>
-      </c>
-      <c r="B145" s="7" t="s">
-        <v>342</v>
       </c>
       <c r="C145" s="1" t="s">
         <v>345</v>
       </c>
       <c r="D145" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E145" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="F145" s="1" t="n">
         <v>0</v>
@@ -5240,20 +5097,20 @@
       </c>
     </row>
     <row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A146" s="1" t="s">
+      <c r="A146" s="7" t="s">
         <v>346</v>
       </c>
       <c r="B146" s="7" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="C146" s="1" t="s">
         <v>347</v>
       </c>
       <c r="D146" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E146" s="1" t="s">
-        <v>348</v>
+        <v>48</v>
       </c>
       <c r="F146" s="1" t="n">
         <v>0</v>
@@ -5264,19 +5121,19 @@
     </row>
     <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A147" s="1" t="s">
+        <v>348</v>
+      </c>
+      <c r="B147" s="7" t="s">
+        <v>344</v>
+      </c>
+      <c r="C147" s="1" t="s">
         <v>349</v>
       </c>
-      <c r="B147" s="7" t="s">
-        <v>342</v>
-      </c>
-      <c r="C147" s="1" t="s">
+      <c r="D147" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E147" s="1" t="s">
         <v>350</v>
-      </c>
-      <c r="D147" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E147" s="1" t="s">
-        <v>351</v>
       </c>
       <c r="F147" s="1" t="n">
         <v>0</v>
@@ -5287,19 +5144,19 @@
     </row>
     <row r="148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A148" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="B148" s="7" t="s">
+        <v>344</v>
+      </c>
+      <c r="C148" s="1" t="s">
         <v>352</v>
       </c>
-      <c r="B148" s="7" t="s">
-        <v>342</v>
-      </c>
-      <c r="C148" s="1" t="s">
+      <c r="D148" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E148" s="1" t="s">
         <v>353</v>
-      </c>
-      <c r="D148" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E148" s="1" t="s">
-        <v>354</v>
       </c>
       <c r="F148" s="1" t="n">
         <v>0</v>
@@ -5310,65 +5167,68 @@
     </row>
     <row r="149" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A149" s="1" t="s">
+        <v>354</v>
+      </c>
+      <c r="B149" s="7" t="s">
+        <v>344</v>
+      </c>
+      <c r="C149" s="1" t="s">
         <v>355</v>
       </c>
-      <c r="B149" s="7" t="s">
-        <v>342</v>
-      </c>
-      <c r="C149" s="1" t="s">
+      <c r="D149" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E149" s="1" t="s">
         <v>356</v>
       </c>
-      <c r="D149" s="1" t="s">
-        <v>45</v>
-      </c>
       <c r="F149" s="1" t="n">
         <v>0</v>
       </c>
+      <c r="G149" s="1" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="150" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A150" s="7" t="s">
+      <c r="A150" s="1" t="s">
         <v>357</v>
       </c>
       <c r="B150" s="7" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="C150" s="1" t="s">
         <v>358</v>
       </c>
       <c r="D150" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E150" s="1" t="s">
-        <v>72</v>
+        <v>47</v>
       </c>
       <c r="F150" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="G150" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H150" s="1" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="151" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A151" s="1" t="s">
+      <c r="A151" s="7" t="s">
         <v>359</v>
       </c>
       <c r="B151" s="7" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="C151" s="1" t="s">
         <v>360</v>
       </c>
       <c r="D151" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E151" s="1" t="s">
-        <v>102</v>
+        <v>74</v>
       </c>
       <c r="F151" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="G151" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H151" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="152" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5376,21 +5236,18 @@
         <v>361</v>
       </c>
       <c r="B152" s="7" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="C152" s="1" t="s">
         <v>362</v>
       </c>
       <c r="D152" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E152" s="1" t="s">
-        <v>193</v>
+        <v>104</v>
       </c>
       <c r="F152" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G152" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5399,48 +5256,48 @@
         <v>363</v>
       </c>
       <c r="B153" s="7" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="C153" s="1" t="s">
         <v>364</v>
       </c>
       <c r="D153" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E153" s="1" t="s">
-        <v>152</v>
+        <v>195</v>
       </c>
       <c r="F153" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G153" s="1" t="n">
         <v>0</v>
-      </c>
-      <c r="H153" s="1" t="n">
-        <v>100</v>
       </c>
     </row>
     <row r="154" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A154" s="1" t="s">
         <v>365</v>
       </c>
-      <c r="B154" s="1" t="s">
-        <v>342</v>
+      <c r="B154" s="7" t="s">
+        <v>344</v>
       </c>
       <c r="C154" s="1" t="s">
         <v>366</v>
       </c>
       <c r="D154" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E154" s="1" t="s">
-        <v>351</v>
+        <v>154</v>
       </c>
       <c r="F154" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G154" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="H154" s="1" t="n">
+        <v>100</v>
       </c>
     </row>
     <row r="155" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5448,16 +5305,16 @@
         <v>367</v>
       </c>
       <c r="B155" s="1" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="C155" s="1" t="s">
         <v>368</v>
       </c>
       <c r="D155" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E155" s="1" t="s">
-        <v>46</v>
+        <v>353</v>
       </c>
       <c r="F155" s="1" t="n">
         <v>0</v>
@@ -5470,17 +5327,17 @@
       <c r="A156" s="1" t="s">
         <v>369</v>
       </c>
-      <c r="B156" s="7" t="s">
-        <v>342</v>
+      <c r="B156" s="1" t="s">
+        <v>344</v>
       </c>
       <c r="C156" s="1" t="s">
         <v>370</v>
       </c>
       <c r="D156" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E156" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="F156" s="1" t="n">
         <v>0</v>
@@ -5494,16 +5351,16 @@
         <v>371</v>
       </c>
       <c r="B157" s="7" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="C157" s="1" t="s">
         <v>372</v>
       </c>
       <c r="D157" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E157" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="F157" s="1" t="n">
         <v>0</v>
@@ -5517,16 +5374,16 @@
         <v>373</v>
       </c>
       <c r="B158" s="7" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="C158" s="1" t="s">
         <v>374</v>
       </c>
       <c r="D158" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E158" s="1" t="s">
-        <v>375</v>
+        <v>48</v>
       </c>
       <c r="F158" s="1" t="n">
         <v>0</v>
@@ -5537,28 +5394,25 @@
     </row>
     <row r="159" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A159" s="1" t="s">
+        <v>375</v>
+      </c>
+      <c r="B159" s="7" t="s">
+        <v>344</v>
+      </c>
+      <c r="C159" s="1" t="s">
         <v>376</v>
       </c>
-      <c r="B159" s="7" t="s">
-        <v>342</v>
-      </c>
-      <c r="C159" s="1" t="s">
+      <c r="D159" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E159" s="1" t="s">
         <v>377</v>
       </c>
-      <c r="D159" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E159" s="1" t="s">
-        <v>152</v>
-      </c>
       <c r="F159" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G159" s="1" t="n">
         <v>0</v>
-      </c>
-      <c r="H159" s="1" t="n">
-        <v>100</v>
       </c>
     </row>
     <row r="160" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5566,16 +5420,16 @@
         <v>378</v>
       </c>
       <c r="B160" s="7" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="C160" s="1" t="s">
         <v>379</v>
       </c>
       <c r="D160" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E160" s="1" t="s">
-        <v>72</v>
+        <v>154</v>
       </c>
       <c r="F160" s="1" t="n">
         <v>0</v>
@@ -5584,7 +5438,7 @@
         <v>0</v>
       </c>
       <c r="H160" s="1" t="n">
-        <v>1</v>
+        <v>100</v>
       </c>
     </row>
     <row r="161" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5592,16 +5446,16 @@
         <v>380</v>
       </c>
       <c r="B161" s="7" t="s">
-        <v>342</v>
-      </c>
-      <c r="C161" s="7" t="s">
+        <v>344</v>
+      </c>
+      <c r="C161" s="1" t="s">
         <v>381</v>
       </c>
       <c r="D161" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E161" s="1" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="F161" s="1" t="n">
         <v>0</v>
@@ -5618,16 +5472,16 @@
         <v>382</v>
       </c>
       <c r="B162" s="7" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="C162" s="7" t="s">
         <v>383</v>
       </c>
       <c r="D162" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E162" s="1" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="F162" s="1" t="n">
         <v>0</v>
@@ -5644,22 +5498,25 @@
         <v>384</v>
       </c>
       <c r="B163" s="7" t="s">
-        <v>342</v>
-      </c>
-      <c r="C163" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="C163" s="7" t="s">
         <v>385</v>
       </c>
       <c r="D163" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E163" s="1" t="s">
-        <v>375</v>
+        <v>74</v>
       </c>
       <c r="F163" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G163" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="H163" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="164" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5667,16 +5524,16 @@
         <v>386</v>
       </c>
       <c r="B164" s="7" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="C164" s="1" t="s">
         <v>387</v>
       </c>
       <c r="D164" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E164" s="1" t="s">
-        <v>46</v>
+        <v>377</v>
       </c>
       <c r="F164" s="1" t="n">
         <v>0</v>
@@ -5685,6 +5542,30 @@
         <v>0</v>
       </c>
     </row>
+    <row r="165" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A165" s="1" t="s">
+        <v>388</v>
+      </c>
+      <c r="B165" s="7" t="s">
+        <v>344</v>
+      </c>
+      <c r="C165" s="1" t="s">
+        <v>389</v>
+      </c>
+      <c r="D165" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E165" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="F165" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G165" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
new parameters in SpParams for phenology
</commit_message>
<xml_diff>
--- a/data-raw/SpParamsDefinition.xlsx
+++ b/data-raw/SpParamsDefinition.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="789" uniqueCount="390">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="799" uniqueCount="394">
   <si>
     <t xml:space="preserve">ParameterName</t>
   </si>
@@ -319,15 +319,21 @@
     <t xml:space="preserve">years</t>
   </si>
   <si>
+    <t xml:space="preserve">BudFormationDays</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Number of days required to complete bud formation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">days</t>
+  </si>
+  <si>
     <t xml:space="preserve">t0gdd</t>
   </si>
   <si>
     <t xml:space="preserve">Date to start the accumulation of degree days</t>
   </si>
   <si>
-    <t xml:space="preserve">days</t>
-  </si>
-  <si>
     <t xml:space="preserve">Sgdd</t>
   </si>
   <si>
@@ -341,6 +347,12 @@
   </si>
   <si>
     <t xml:space="preserve">Base temperature for the calculation of degree days to leaf budburst</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ugdd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Degree days to complete leaf unfolding after budburst has occurred</t>
   </si>
   <si>
     <t xml:space="preserve">Ssen</t>
@@ -1955,7 +1967,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H1048576"/>
+  <dimension ref="A1:H167"/>
   <sheetFormatPr defaultColWidth="10.25" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="25.25"/>
@@ -2834,7 +2846,7 @@
         <v>100</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>47</v>
+        <v>14</v>
       </c>
       <c r="E46" s="5" t="s">
         <v>101</v>
@@ -2844,9 +2856,6 @@
       </c>
       <c r="G46" s="1" t="n">
         <v>0</v>
-      </c>
-      <c r="H46" s="1" t="n">
-        <v>365</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2863,32 +2872,38 @@
         <v>47</v>
       </c>
       <c r="E47" s="5" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="F47" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G47" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="H47" s="1" t="n">
+        <v>365</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="3" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B48" s="6" t="s">
         <v>96</v>
       </c>
       <c r="C48" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="D48" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E48" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="D48" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="E48" s="5" t="s">
-        <v>104</v>
-      </c>
       <c r="F48" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G48" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2906,7 +2921,7 @@
         <v>47</v>
       </c>
       <c r="E49" s="5" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="F49" s="1" t="n">
         <v>0</v>
@@ -2926,145 +2941,148 @@
         <v>47</v>
       </c>
       <c r="E50" s="5" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="F50" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G50" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B51" s="6" t="s">
         <v>96</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D51" s="1" t="s">
         <v>47</v>
       </c>
       <c r="E51" s="5" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="F51" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G51" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B52" s="6" t="s">
         <v>96</v>
       </c>
       <c r="C52" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="D52" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E52" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="D52" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="E52" s="5" t="s">
-        <v>116</v>
-      </c>
       <c r="F52" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G52" s="1" t="n">
         <v>0</v>
-      </c>
-      <c r="H52" s="1" t="n">
-        <v>2</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="3" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B53" s="6" t="s">
         <v>96</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>14</v>
+        <v>47</v>
       </c>
       <c r="E53" s="5" t="s">
-        <v>116</v>
+        <v>106</v>
       </c>
       <c r="F53" s="1" t="n">
         <v>0</v>
-      </c>
-      <c r="G53" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H53" s="1" t="n">
-        <v>2</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="B54" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="C54" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="B54" s="6" t="s">
+      <c r="D54" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E54" s="5" t="s">
         <v>120</v>
       </c>
-      <c r="C54" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="D54" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="E54" s="5" t="s">
-        <v>122</v>
-      </c>
       <c r="F54" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G54" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="H54" s="1" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="3" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="B55" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="C55" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="D55" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E55" s="5" t="s">
         <v>120</v>
       </c>
-      <c r="C55" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="D55" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="E55" s="1" t="s">
-        <v>125</v>
-      </c>
       <c r="F55" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G55" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="H55" s="1" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="B56" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="C56" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="D56" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E56" s="5" t="s">
         <v>126</v>
-      </c>
-      <c r="B56" s="6" t="s">
-        <v>120</v>
-      </c>
-      <c r="C56" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="D56" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="E56" s="1" t="s">
-        <v>125</v>
       </c>
       <c r="F56" s="1" t="n">
         <v>0</v>
@@ -3075,19 +3093,19 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="B57" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="C57" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="B57" s="6" t="s">
-        <v>120</v>
-      </c>
-      <c r="C57" s="1" t="s">
+      <c r="D57" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E57" s="1" t="s">
         <v>129</v>
-      </c>
-      <c r="D57" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="E57" s="1" t="s">
-        <v>125</v>
       </c>
       <c r="F57" s="1" t="n">
         <v>0</v>
@@ -3101,7 +3119,7 @@
         <v>130</v>
       </c>
       <c r="B58" s="6" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="C58" s="1" t="s">
         <v>131</v>
@@ -3110,56 +3128,53 @@
         <v>47</v>
       </c>
       <c r="E58" s="1" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="F58" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G58" s="1" t="n">
         <v>0</v>
-      </c>
-      <c r="H58" s="1" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="B59" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="C59" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="B59" s="6" t="s">
-        <v>120</v>
-      </c>
-      <c r="C59" s="1" t="s">
-        <v>134</v>
-      </c>
       <c r="D59" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="E59" s="5" t="s">
-        <v>135</v>
+      <c r="E59" s="1" t="s">
+        <v>129</v>
       </c>
       <c r="F59" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G59" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="B60" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="C60" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="D60" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E60" s="1" t="s">
         <v>136</v>
-      </c>
-      <c r="B60" s="6" t="s">
-        <v>120</v>
-      </c>
-      <c r="C60" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="D60" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="E60" s="5" t="s">
-        <v>132</v>
       </c>
       <c r="F60" s="1" t="n">
         <v>0</v>
@@ -3173,65 +3188,68 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="B61" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="C61" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="B61" s="6" t="s">
-        <v>120</v>
-      </c>
-      <c r="C61" s="1" t="s">
+      <c r="D61" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E61" s="5" t="s">
         <v>139</v>
       </c>
-      <c r="D61" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="E61" s="1" t="s">
-        <v>140</v>
-      </c>
       <c r="F61" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G61" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="B62" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="C62" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="B62" s="6" t="s">
-        <v>120</v>
-      </c>
-      <c r="C62" s="1" t="s">
-        <v>142</v>
-      </c>
       <c r="D62" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="E62" s="7" t="s">
-        <v>140</v>
+      <c r="E62" s="5" t="s">
+        <v>136</v>
       </c>
       <c r="F62" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G62" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="H62" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="B63" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="C63" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="B63" s="6" t="s">
-        <v>120</v>
-      </c>
-      <c r="C63" s="1" t="s">
+      <c r="D63" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E63" s="1" t="s">
         <v>144</v>
-      </c>
-      <c r="D63" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="E63" s="1" t="s">
-        <v>48</v>
       </c>
       <c r="F63" s="1" t="n">
         <v>0</v>
@@ -3245,7 +3263,7 @@
         <v>145</v>
       </c>
       <c r="B64" s="6" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="C64" s="1" t="s">
         <v>146</v>
@@ -3253,8 +3271,8 @@
       <c r="D64" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="E64" s="1" t="s">
-        <v>147</v>
+      <c r="E64" s="7" t="s">
+        <v>144</v>
       </c>
       <c r="F64" s="1" t="n">
         <v>0</v>
@@ -3265,19 +3283,19 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="B65" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="C65" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="B65" s="6" t="s">
-        <v>120</v>
-      </c>
-      <c r="C65" s="1" t="s">
-        <v>149</v>
-      </c>
       <c r="D65" s="1" t="s">
         <v>47</v>
       </c>
       <c r="E65" s="1" t="s">
-        <v>150</v>
+        <v>48</v>
       </c>
       <c r="F65" s="1" t="n">
         <v>0</v>
@@ -3288,19 +3306,19 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="B66" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="C66" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="D66" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E66" s="1" t="s">
         <v>151</v>
-      </c>
-      <c r="B66" s="6" t="s">
-        <v>152</v>
-      </c>
-      <c r="C66" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="D66" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="E66" s="5" t="s">
-        <v>154</v>
       </c>
       <c r="F66" s="1" t="n">
         <v>0</v>
@@ -3311,18 +3329,18 @@
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="3" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="B67" s="6" t="s">
-        <v>152</v>
+        <v>124</v>
       </c>
       <c r="C67" s="1" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="D67" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="E67" s="5" t="s">
+      <c r="E67" s="1" t="s">
         <v>154</v>
       </c>
       <c r="F67" s="1" t="n">
@@ -3334,70 +3352,70 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="B68" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="C68" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="B68" s="6" t="s">
-        <v>152</v>
-      </c>
-      <c r="C68" s="1" t="s">
+      <c r="D68" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E68" s="5" t="s">
         <v>158</v>
       </c>
-      <c r="D68" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="E68" s="5" t="s">
-        <v>159</v>
-      </c>
       <c r="F68" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="H68" s="1" t="n">
+      <c r="G68" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="B69" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="C69" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="B69" s="6" t="s">
-        <v>152</v>
-      </c>
-      <c r="C69" s="1" t="s">
-        <v>161</v>
-      </c>
       <c r="D69" s="1" t="s">
         <v>47</v>
       </c>
       <c r="E69" s="5" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="F69" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="H69" s="1" t="n">
+      <c r="G69" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="B70" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="C70" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="B70" s="6" t="s">
-        <v>152</v>
-      </c>
-      <c r="C70" s="1" t="s">
+      <c r="D70" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E70" s="5" t="s">
         <v>163</v>
       </c>
-      <c r="D70" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="E70" s="5" t="s">
-        <v>159</v>
-      </c>
       <c r="F70" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="G70" s="1" t="n">
+      <c r="H70" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3406,7 +3424,7 @@
         <v>164</v>
       </c>
       <c r="B71" s="6" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="C71" s="1" t="s">
         <v>165</v>
@@ -3415,16 +3433,13 @@
         <v>47</v>
       </c>
       <c r="E71" s="5" t="s">
-        <v>132</v>
+        <v>163</v>
       </c>
       <c r="F71" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="G71" s="1" t="n">
-        <v>0</v>
-      </c>
       <c r="H71" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3432,7 +3447,7 @@
         <v>166</v>
       </c>
       <c r="B72" s="6" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="C72" s="1" t="s">
         <v>167</v>
@@ -3441,12 +3456,12 @@
         <v>47</v>
       </c>
       <c r="E72" s="5" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="F72" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="H72" s="1" t="n">
+      <c r="G72" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3455,7 +3470,7 @@
         <v>168</v>
       </c>
       <c r="B73" s="6" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="C73" s="1" t="s">
         <v>169</v>
@@ -3464,13 +3479,16 @@
         <v>47</v>
       </c>
       <c r="E73" s="5" t="s">
-        <v>159</v>
+        <v>136</v>
       </c>
       <c r="F73" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G73" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="H73" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3478,7 +3496,7 @@
         <v>170</v>
       </c>
       <c r="B74" s="6" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="C74" s="1" t="s">
         <v>171</v>
@@ -3487,16 +3505,13 @@
         <v>47</v>
       </c>
       <c r="E74" s="5" t="s">
-        <v>132</v>
+        <v>163</v>
       </c>
       <c r="F74" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="G74" s="1" t="n">
-        <v>0</v>
-      </c>
       <c r="H74" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3504,16 +3519,16 @@
         <v>172</v>
       </c>
       <c r="B75" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="C75" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="C75" s="1" t="s">
-        <v>174</v>
-      </c>
       <c r="D75" s="1" t="s">
         <v>47</v>
       </c>
       <c r="E75" s="5" t="s">
-        <v>175</v>
+        <v>163</v>
       </c>
       <c r="F75" s="1" t="n">
         <v>0</v>
@@ -3524,42 +3539,45 @@
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="3" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="B76" s="6" t="s">
-        <v>173</v>
+        <v>156</v>
       </c>
       <c r="C76" s="1" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="D76" s="1" t="s">
         <v>47</v>
       </c>
       <c r="E76" s="5" t="s">
-        <v>178</v>
+        <v>136</v>
       </c>
       <c r="F76" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G76" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="H76" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="B77" s="6" t="s">
+        <v>177</v>
+      </c>
+      <c r="C77" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="D77" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E77" s="5" t="s">
         <v>179</v>
-      </c>
-      <c r="B77" s="6" t="s">
-        <v>173</v>
-      </c>
-      <c r="C77" s="1" t="s">
-        <v>180</v>
-      </c>
-      <c r="D77" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="E77" s="5" t="s">
-        <v>154</v>
       </c>
       <c r="F77" s="1" t="n">
         <v>0</v>
@@ -3570,19 +3588,19 @@
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="B78" s="6" t="s">
+        <v>177</v>
+      </c>
+      <c r="C78" s="1" t="s">
         <v>181</v>
       </c>
-      <c r="B78" s="6" t="s">
-        <v>173</v>
-      </c>
-      <c r="C78" s="1" t="s">
+      <c r="D78" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E78" s="5" t="s">
         <v>182</v>
-      </c>
-      <c r="D78" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="E78" s="5" t="s">
-        <v>154</v>
       </c>
       <c r="F78" s="1" t="n">
         <v>0</v>
@@ -3596,7 +3614,7 @@
         <v>183</v>
       </c>
       <c r="B79" s="6" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="C79" s="1" t="s">
         <v>184</v>
@@ -3605,7 +3623,7 @@
         <v>47</v>
       </c>
       <c r="E79" s="5" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="F79" s="1" t="n">
         <v>0</v>
@@ -3619,42 +3637,39 @@
         <v>185</v>
       </c>
       <c r="B80" s="6" t="s">
+        <v>177</v>
+      </c>
+      <c r="C80" s="1" t="s">
         <v>186</v>
       </c>
-      <c r="C80" s="1" t="s">
-        <v>187</v>
-      </c>
       <c r="D80" s="1" t="s">
         <v>47</v>
       </c>
       <c r="E80" s="5" t="s">
-        <v>188</v>
+        <v>158</v>
       </c>
       <c r="F80" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G80" s="1" t="n">
         <v>0</v>
-      </c>
-      <c r="H80" s="1" t="n">
-        <v>90</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="3" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="B81" s="6" t="s">
-        <v>186</v>
+        <v>177</v>
       </c>
       <c r="C81" s="1" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="D81" s="1" t="s">
         <v>47</v>
       </c>
       <c r="E81" s="5" t="s">
-        <v>188</v>
+        <v>158</v>
       </c>
       <c r="F81" s="1" t="n">
         <v>0</v>
@@ -3665,25 +3680,28 @@
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="B82" s="6" t="s">
+        <v>190</v>
+      </c>
+      <c r="C82" s="1" t="s">
         <v>191</v>
       </c>
-      <c r="B82" s="6" t="s">
-        <v>186</v>
-      </c>
-      <c r="C82" s="1" t="s">
+      <c r="D82" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E82" s="5" t="s">
         <v>192</v>
       </c>
-      <c r="D82" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="E82" s="5" t="s">
-        <v>74</v>
-      </c>
       <c r="F82" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G82" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="H82" s="1" t="n">
+        <v>90</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3691,7 +3709,7 @@
         <v>193</v>
       </c>
       <c r="B83" s="6" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="C83" s="1" t="s">
         <v>194</v>
@@ -3700,7 +3718,7 @@
         <v>47</v>
       </c>
       <c r="E83" s="5" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="F83" s="1" t="n">
         <v>0</v>
@@ -3711,19 +3729,19 @@
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="B84" s="6" t="s">
+        <v>190</v>
+      </c>
+      <c r="C84" s="1" t="s">
         <v>196</v>
       </c>
-      <c r="B84" s="6" t="s">
-        <v>186</v>
-      </c>
-      <c r="C84" s="1" t="s">
-        <v>197</v>
-      </c>
       <c r="D84" s="1" t="s">
         <v>47</v>
       </c>
       <c r="E84" s="5" t="s">
-        <v>195</v>
+        <v>74</v>
       </c>
       <c r="F84" s="1" t="n">
         <v>0</v>
@@ -3734,19 +3752,19 @@
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="3" t="s">
+        <v>197</v>
+      </c>
+      <c r="B85" s="6" t="s">
+        <v>190</v>
+      </c>
+      <c r="C85" s="1" t="s">
         <v>198</v>
       </c>
-      <c r="B85" s="6" t="s">
-        <v>186</v>
-      </c>
-      <c r="C85" s="1" t="s">
+      <c r="D85" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E85" s="5" t="s">
         <v>199</v>
-      </c>
-      <c r="D85" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="E85" s="5" t="s">
-        <v>195</v>
       </c>
       <c r="F85" s="1" t="n">
         <v>0</v>
@@ -3760,7 +3778,7 @@
         <v>200</v>
       </c>
       <c r="B86" s="6" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="C86" s="1" t="s">
         <v>201</v>
@@ -3769,7 +3787,7 @@
         <v>47</v>
       </c>
       <c r="E86" s="5" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="F86" s="1" t="n">
         <v>0</v>
@@ -3780,46 +3798,56 @@
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="B87" s="6" t="s">
+        <v>190</v>
+      </c>
+      <c r="C87" s="1" t="s">
         <v>203</v>
       </c>
-      <c r="B87" s="6" t="s">
-        <v>204</v>
-      </c>
-      <c r="C87" s="1" t="s">
-        <v>205</v>
-      </c>
       <c r="D87" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="E87" s="5"/>
+      <c r="E87" s="5" t="s">
+        <v>199</v>
+      </c>
       <c r="F87" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G87" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="3" t="s">
+        <v>204</v>
+      </c>
+      <c r="B88" s="6" t="s">
+        <v>190</v>
+      </c>
+      <c r="C88" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="D88" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E88" s="5" t="s">
         <v>206</v>
       </c>
-      <c r="B88" s="6" t="s">
-        <v>204</v>
-      </c>
-      <c r="C88" s="1" t="s">
-        <v>207</v>
-      </c>
-      <c r="D88" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="E88" s="5"/>
       <c r="F88" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G88" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="3" t="s">
+        <v>207</v>
+      </c>
+      <c r="B89" s="6" t="s">
         <v>208</v>
-      </c>
-      <c r="B89" s="6" t="s">
-        <v>204</v>
       </c>
       <c r="C89" s="1" t="s">
         <v>209</v>
@@ -3827,25 +3855,20 @@
       <c r="D89" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="E89" s="5" t="s">
-        <v>210</v>
-      </c>
+      <c r="E89" s="5"/>
       <c r="F89" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H89" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="3" t="s">
+        <v>210</v>
+      </c>
+      <c r="B90" s="6" t="s">
+        <v>208</v>
+      </c>
+      <c r="C90" s="1" t="s">
         <v>211</v>
-      </c>
-      <c r="B90" s="6" t="s">
-        <v>204</v>
-      </c>
-      <c r="C90" s="1" t="s">
-        <v>212</v>
       </c>
       <c r="D90" s="1" t="s">
         <v>47</v>
@@ -3854,42 +3877,39 @@
       <c r="F90" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="G90" s="1" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="3" t="s">
+        <v>212</v>
+      </c>
+      <c r="B91" s="6" t="s">
+        <v>208</v>
+      </c>
+      <c r="C91" s="1" t="s">
         <v>213</v>
       </c>
-      <c r="B91" s="6" t="s">
-        <v>204</v>
-      </c>
-      <c r="C91" s="1" t="s">
+      <c r="D91" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E91" s="5" t="s">
         <v>214</v>
       </c>
-      <c r="D91" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="E91" s="5" t="s">
-        <v>215</v>
-      </c>
       <c r="F91" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="G91" s="1" t="n">
+      <c r="H91" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="B92" s="6" t="s">
+        <v>208</v>
+      </c>
+      <c r="C92" s="1" t="s">
         <v>216</v>
-      </c>
-      <c r="B92" s="6" t="s">
-        <v>204</v>
-      </c>
-      <c r="C92" s="1" t="s">
-        <v>217</v>
       </c>
       <c r="D92" s="1" t="s">
         <v>47</v>
@@ -3898,22 +3918,30 @@
       <c r="F92" s="1" t="n">
         <v>0</v>
       </c>
+      <c r="G92" s="1" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="3" t="s">
+        <v>217</v>
+      </c>
+      <c r="B93" s="6" t="s">
+        <v>208</v>
+      </c>
+      <c r="C93" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="B93" s="6" t="s">
-        <v>204</v>
-      </c>
-      <c r="C93" s="1" t="s">
+      <c r="D93" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E93" s="5" t="s">
         <v>219</v>
       </c>
-      <c r="D93" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="E93" s="5"/>
       <c r="F93" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G93" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3922,7 +3950,7 @@
         <v>220</v>
       </c>
       <c r="B94" s="6" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="C94" s="1" t="s">
         <v>221</v>
@@ -3935,78 +3963,71 @@
         <v>0</v>
       </c>
     </row>
-    <row r="95" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="3" t="s">
         <v>222</v>
       </c>
       <c r="B95" s="6" t="s">
-        <v>204</v>
-      </c>
-      <c r="C95" s="8" t="s">
+        <v>208</v>
+      </c>
+      <c r="C95" s="1" t="s">
         <v>223</v>
       </c>
       <c r="D95" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="E95" s="5" t="s">
-        <v>224</v>
-      </c>
+      <c r="E95" s="5"/>
       <c r="F95" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G95" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="3" t="s">
+        <v>224</v>
+      </c>
+      <c r="B96" s="6" t="s">
+        <v>208</v>
+      </c>
+      <c r="C96" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="B96" s="6" t="s">
-        <v>204</v>
-      </c>
-      <c r="C96" s="1" t="s">
+      <c r="D96" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E96" s="5"/>
+      <c r="F96" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="97" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A97" s="3" t="s">
         <v>226</v>
       </c>
-      <c r="D96" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="E96" s="5" t="s">
-        <v>224</v>
-      </c>
-      <c r="F96" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G96" s="1" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A97" s="3" t="s">
+      <c r="B97" s="6" t="s">
+        <v>208</v>
+      </c>
+      <c r="C97" s="8" t="s">
         <v>227</v>
       </c>
-      <c r="B97" s="6" t="s">
-        <v>204</v>
-      </c>
-      <c r="C97" s="1" t="s">
+      <c r="D97" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E97" s="5" t="s">
         <v>228</v>
       </c>
-      <c r="D97" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="E97" s="5" t="s">
-        <v>104</v>
-      </c>
       <c r="F97" s="1" t="n">
         <v>0</v>
       </c>
-    </row>
-    <row r="98" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G97" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="3" t="s">
         <v>229</v>
       </c>
       <c r="B98" s="6" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="C98" s="1" t="s">
         <v>230</v>
@@ -4014,17 +4035,22 @@
       <c r="D98" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="E98" s="5"/>
+      <c r="E98" s="5" t="s">
+        <v>228</v>
+      </c>
       <c r="F98" s="1" t="n">
         <v>0</v>
       </c>
-    </row>
-    <row r="99" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G98" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="3" t="s">
         <v>231</v>
       </c>
       <c r="B99" s="6" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="C99" s="1" t="s">
         <v>232</v>
@@ -4033,137 +4059,129 @@
         <v>47</v>
       </c>
       <c r="E99" s="5" t="s">
-        <v>233</v>
+        <v>106</v>
       </c>
       <c r="F99" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G99" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="B100" s="6" t="s">
+        <v>208</v>
+      </c>
+      <c r="C100" s="1" t="s">
         <v>234</v>
       </c>
-      <c r="B100" s="6" t="s">
-        <v>204</v>
-      </c>
-      <c r="C100" s="1" t="s">
-        <v>235</v>
-      </c>
       <c r="D100" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="E100" s="5" t="s">
-        <v>210</v>
-      </c>
+      <c r="E100" s="5"/>
       <c r="F100" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H100" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="B101" s="6" t="s">
+        <v>208</v>
+      </c>
+      <c r="C101" s="1" t="s">
         <v>236</v>
       </c>
-      <c r="B101" s="6" t="s">
-        <v>204</v>
-      </c>
-      <c r="C101" s="1" t="s">
+      <c r="D101" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E101" s="5" t="s">
         <v>237</v>
       </c>
-      <c r="D101" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="E101" s="5" t="s">
-        <v>238</v>
-      </c>
       <c r="F101" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G101" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="H101" s="1"/>
     </row>
     <row r="102" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="3" t="s">
+        <v>238</v>
+      </c>
+      <c r="B102" s="6" t="s">
+        <v>208</v>
+      </c>
+      <c r="C102" s="1" t="s">
         <v>239</v>
       </c>
-      <c r="B102" s="6" t="s">
-        <v>204</v>
-      </c>
-      <c r="C102" s="1" t="s">
+      <c r="D102" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E102" s="5" t="s">
+        <v>214</v>
+      </c>
+      <c r="F102" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H102" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="103" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A103" s="3" t="s">
         <v>240</v>
       </c>
-      <c r="D102" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="E102" s="5" t="s">
+      <c r="B103" s="6" t="s">
+        <v>208</v>
+      </c>
+      <c r="C103" s="1" t="s">
         <v>241</v>
       </c>
-      <c r="F102" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G102" s="1" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A103" s="3" t="s">
+      <c r="D103" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E103" s="5" t="s">
         <v>242</v>
       </c>
-      <c r="B103" s="6" t="s">
-        <v>204</v>
-      </c>
-      <c r="C103" s="1" t="s">
-        <v>243</v>
-      </c>
-      <c r="D103" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="E103" s="5" t="s">
-        <v>210</v>
-      </c>
       <c r="F103" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="H103" s="1" t="n">
-        <v>0</v>
-      </c>
+      <c r="G103" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H103" s="1"/>
     </row>
     <row r="104" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="3" t="s">
+        <v>243</v>
+      </c>
+      <c r="B104" s="6" t="s">
+        <v>208</v>
+      </c>
+      <c r="C104" s="1" t="s">
         <v>244</v>
       </c>
-      <c r="B104" s="6" t="s">
-        <v>204</v>
-      </c>
-      <c r="C104" s="1" t="s">
+      <c r="D104" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E104" s="5" t="s">
         <v>245</v>
       </c>
-      <c r="D104" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="E104" s="5" t="s">
-        <v>210</v>
-      </c>
       <c r="F104" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="H104" s="1" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="105" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G104" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="3" t="s">
         <v>246</v>
       </c>
       <c r="B105" s="6" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="C105" s="1" t="s">
         <v>247</v>
@@ -4172,7 +4190,7 @@
         <v>47</v>
       </c>
       <c r="E105" s="5" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="F105" s="1" t="n">
         <v>0</v>
@@ -4181,12 +4199,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="106" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="3" t="s">
         <v>248</v>
       </c>
       <c r="B106" s="6" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="C106" s="1" t="s">
         <v>249</v>
@@ -4195,22 +4213,21 @@
         <v>47</v>
       </c>
       <c r="E106" s="5" t="s">
-        <v>238</v>
+        <v>214</v>
       </c>
       <c r="F106" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="G106" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H106" s="1"/>
-    </row>
-    <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="H106" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="107" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="3" t="s">
         <v>250</v>
       </c>
       <c r="B107" s="6" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="C107" s="1" t="s">
         <v>251</v>
@@ -4219,7 +4236,7 @@
         <v>47</v>
       </c>
       <c r="E107" s="5" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="F107" s="1" t="n">
         <v>0</v>
@@ -4228,12 +4245,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="108" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="3" t="s">
         <v>252</v>
       </c>
       <c r="B108" s="6" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="C108" s="1" t="s">
         <v>253</v>
@@ -4242,21 +4259,22 @@
         <v>47</v>
       </c>
       <c r="E108" s="5" t="s">
-        <v>210</v>
+        <v>242</v>
       </c>
       <c r="F108" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="H108" s="1" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="109" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G108" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H108" s="1"/>
+    </row>
+    <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="3" t="s">
         <v>254</v>
       </c>
       <c r="B109" s="6" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="C109" s="1" t="s">
         <v>255</v>
@@ -4265,7 +4283,7 @@
         <v>47</v>
       </c>
       <c r="E109" s="5" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="F109" s="1" t="n">
         <v>0</v>
@@ -4274,12 +4292,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="110" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="3" t="s">
         <v>256</v>
       </c>
       <c r="B110" s="6" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="C110" s="1" t="s">
         <v>257</v>
@@ -4288,22 +4306,21 @@
         <v>47</v>
       </c>
       <c r="E110" s="5" t="s">
-        <v>238</v>
+        <v>214</v>
       </c>
       <c r="F110" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="G110" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H110" s="1"/>
-    </row>
-    <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="H110" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="111" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A111" s="3" t="s">
         <v>258</v>
       </c>
       <c r="B111" s="6" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="C111" s="1" t="s">
         <v>259</v>
@@ -4312,58 +4329,59 @@
         <v>47</v>
       </c>
       <c r="E111" s="5" t="s">
-        <v>260</v>
+        <v>214</v>
       </c>
       <c r="F111" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="G111" s="1" t="n">
+      <c r="H111" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="3" t="s">
+        <v>260</v>
+      </c>
+      <c r="B112" s="6" t="s">
+        <v>208</v>
+      </c>
+      <c r="C112" s="1" t="s">
         <v>261</v>
       </c>
-      <c r="B112" s="6" t="s">
-        <v>204</v>
-      </c>
-      <c r="C112" s="1" t="s">
-        <v>262</v>
-      </c>
       <c r="D112" s="1" t="s">
         <v>47</v>
       </c>
       <c r="E112" s="5" t="s">
-        <v>210</v>
+        <v>242</v>
       </c>
       <c r="F112" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="H112" s="1" t="n">
-        <v>0</v>
-      </c>
+      <c r="G112" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H112" s="1"/>
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A113" s="3" t="s">
+        <v>262</v>
+      </c>
+      <c r="B113" s="6" t="s">
+        <v>208</v>
+      </c>
+      <c r="C113" s="1" t="s">
         <v>263</v>
       </c>
-      <c r="B113" s="6" t="s">
-        <v>204</v>
-      </c>
-      <c r="C113" s="1" t="s">
+      <c r="D113" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E113" s="5" t="s">
         <v>264</v>
       </c>
-      <c r="D113" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="E113" s="5" t="s">
-        <v>210</v>
-      </c>
       <c r="F113" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="H113" s="1" t="n">
+      <c r="G113" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4372,7 +4390,7 @@
         <v>265</v>
       </c>
       <c r="B114" s="6" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="C114" s="1" t="s">
         <v>266</v>
@@ -4381,7 +4399,7 @@
         <v>47</v>
       </c>
       <c r="E114" s="5" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="F114" s="1" t="n">
         <v>0</v>
@@ -4395,7 +4413,7 @@
         <v>267</v>
       </c>
       <c r="B115" s="6" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="C115" s="1" t="s">
         <v>268</v>
@@ -4404,22 +4422,21 @@
         <v>47</v>
       </c>
       <c r="E115" s="5" t="s">
-        <v>238</v>
+        <v>214</v>
       </c>
       <c r="F115" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="G115" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H115" s="1"/>
+      <c r="H115" s="1" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A116" s="3" t="s">
         <v>269</v>
       </c>
       <c r="B116" s="6" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="C116" s="1" t="s">
         <v>270</v>
@@ -4428,12 +4445,12 @@
         <v>47</v>
       </c>
       <c r="E116" s="5" t="s">
-        <v>260</v>
+        <v>214</v>
       </c>
       <c r="F116" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="G116" s="1" t="n">
+      <c r="H116" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4442,7 +4459,7 @@
         <v>271</v>
       </c>
       <c r="B117" s="6" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="C117" s="1" t="s">
         <v>272</v>
@@ -4451,21 +4468,22 @@
         <v>47</v>
       </c>
       <c r="E117" s="5" t="s">
-        <v>210</v>
+        <v>242</v>
       </c>
       <c r="F117" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="H117" s="1" t="n">
-        <v>0</v>
-      </c>
+      <c r="G117" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H117" s="1"/>
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A118" s="3" t="s">
         <v>273</v>
       </c>
       <c r="B118" s="6" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="C118" s="1" t="s">
         <v>274</v>
@@ -4474,12 +4492,12 @@
         <v>47</v>
       </c>
       <c r="E118" s="5" t="s">
-        <v>210</v>
+        <v>264</v>
       </c>
       <c r="F118" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="H118" s="1" t="n">
+      <c r="G118" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4488,7 +4506,7 @@
         <v>275</v>
       </c>
       <c r="B119" s="6" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="C119" s="1" t="s">
         <v>276</v>
@@ -4497,7 +4515,7 @@
         <v>47</v>
       </c>
       <c r="E119" s="5" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="F119" s="1" t="n">
         <v>0</v>
@@ -4511,7 +4529,7 @@
         <v>277</v>
       </c>
       <c r="B120" s="6" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="C120" s="1" t="s">
         <v>278</v>
@@ -4520,22 +4538,21 @@
         <v>47</v>
       </c>
       <c r="E120" s="5" t="s">
-        <v>238</v>
+        <v>214</v>
       </c>
       <c r="F120" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="G120" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H120" s="1"/>
+      <c r="H120" s="1" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A121" s="3" t="s">
         <v>279</v>
       </c>
       <c r="B121" s="6" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="C121" s="1" t="s">
         <v>280</v>
@@ -4543,31 +4560,31 @@
       <c r="D121" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="E121" s="9" t="s">
-        <v>281</v>
+      <c r="E121" s="5" t="s">
+        <v>214</v>
       </c>
       <c r="F121" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="G121" s="1" t="n">
+      <c r="H121" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A122" s="3" t="s">
+        <v>281</v>
+      </c>
+      <c r="B122" s="6" t="s">
+        <v>208</v>
+      </c>
+      <c r="C122" s="1" t="s">
         <v>282</v>
       </c>
-      <c r="B122" s="6" t="s">
-        <v>204</v>
-      </c>
-      <c r="C122" s="1" t="s">
-        <v>283</v>
-      </c>
       <c r="D122" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="E122" s="9" t="s">
-        <v>284</v>
+      <c r="E122" s="5" t="s">
+        <v>242</v>
       </c>
       <c r="F122" s="1" t="n">
         <v>0</v>
@@ -4575,22 +4592,23 @@
       <c r="G122" s="1" t="n">
         <v>0</v>
       </c>
+      <c r="H122" s="1"/>
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A123" s="3" t="s">
+        <v>283</v>
+      </c>
+      <c r="B123" s="6" t="s">
+        <v>208</v>
+      </c>
+      <c r="C123" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="D123" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E123" s="9" t="s">
         <v>285</v>
-      </c>
-      <c r="B123" s="6" t="s">
-        <v>204</v>
-      </c>
-      <c r="C123" s="1" t="s">
-        <v>286</v>
-      </c>
-      <c r="D123" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="E123" s="1" t="s">
-        <v>287</v>
       </c>
       <c r="F123" s="1" t="n">
         <v>0</v>
@@ -4601,19 +4619,19 @@
     </row>
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A124" s="3" t="s">
+        <v>286</v>
+      </c>
+      <c r="B124" s="6" t="s">
+        <v>208</v>
+      </c>
+      <c r="C124" s="1" t="s">
+        <v>287</v>
+      </c>
+      <c r="D124" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E124" s="9" t="s">
         <v>288</v>
-      </c>
-      <c r="B124" s="3" t="s">
-        <v>289</v>
-      </c>
-      <c r="C124" s="1" t="s">
-        <v>290</v>
-      </c>
-      <c r="D124" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="E124" s="1" t="s">
-        <v>287</v>
       </c>
       <c r="F124" s="1" t="n">
         <v>0</v>
@@ -4624,19 +4642,19 @@
     </row>
     <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A125" s="3" t="s">
+        <v>289</v>
+      </c>
+      <c r="B125" s="6" t="s">
+        <v>208</v>
+      </c>
+      <c r="C125" s="1" t="s">
+        <v>290</v>
+      </c>
+      <c r="D125" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E125" s="1" t="s">
         <v>291</v>
-      </c>
-      <c r="B125" s="3" t="s">
-        <v>289</v>
-      </c>
-      <c r="C125" s="1" t="s">
-        <v>292</v>
-      </c>
-      <c r="D125" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="E125" s="1" t="s">
-        <v>287</v>
       </c>
       <c r="F125" s="1" t="n">
         <v>0</v>
@@ -4647,10 +4665,10 @@
     </row>
     <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A126" s="3" t="s">
+        <v>292</v>
+      </c>
+      <c r="B126" s="3" t="s">
         <v>293</v>
-      </c>
-      <c r="B126" s="3" t="s">
-        <v>289</v>
       </c>
       <c r="C126" s="1" t="s">
         <v>294</v>
@@ -4659,7 +4677,7 @@
         <v>47</v>
       </c>
       <c r="E126" s="1" t="s">
-        <v>295</v>
+        <v>291</v>
       </c>
       <c r="F126" s="1" t="n">
         <v>0</v>
@@ -4670,19 +4688,19 @@
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A127" s="3" t="s">
+        <v>295</v>
+      </c>
+      <c r="B127" s="3" t="s">
+        <v>293</v>
+      </c>
+      <c r="C127" s="1" t="s">
         <v>296</v>
       </c>
-      <c r="B127" s="3" t="s">
-        <v>289</v>
-      </c>
-      <c r="C127" s="1" t="s">
-        <v>297</v>
-      </c>
       <c r="D127" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="E127" s="7" t="s">
-        <v>298</v>
+      <c r="E127" s="1" t="s">
+        <v>291</v>
       </c>
       <c r="F127" s="1" t="n">
         <v>0</v>
@@ -4693,19 +4711,19 @@
     </row>
     <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A128" s="3" t="s">
+        <v>297</v>
+      </c>
+      <c r="B128" s="3" t="s">
+        <v>293</v>
+      </c>
+      <c r="C128" s="1" t="s">
+        <v>298</v>
+      </c>
+      <c r="D128" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E128" s="1" t="s">
         <v>299</v>
-      </c>
-      <c r="B128" s="3" t="s">
-        <v>289</v>
-      </c>
-      <c r="C128" s="1" t="s">
-        <v>300</v>
-      </c>
-      <c r="D128" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="E128" s="7" t="s">
-        <v>298</v>
       </c>
       <c r="F128" s="1" t="n">
         <v>0</v>
@@ -4716,19 +4734,19 @@
     </row>
     <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A129" s="3" t="s">
+        <v>300</v>
+      </c>
+      <c r="B129" s="3" t="s">
+        <v>293</v>
+      </c>
+      <c r="C129" s="1" t="s">
         <v>301</v>
       </c>
-      <c r="B129" s="3" t="s">
-        <v>289</v>
-      </c>
-      <c r="C129" s="1" t="s">
+      <c r="D129" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E129" s="7" t="s">
         <v>302</v>
-      </c>
-      <c r="D129" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="E129" s="7" t="s">
-        <v>298</v>
       </c>
       <c r="F129" s="1" t="n">
         <v>0</v>
@@ -4742,7 +4760,7 @@
         <v>303</v>
       </c>
       <c r="B130" s="3" t="s">
-        <v>289</v>
+        <v>293</v>
       </c>
       <c r="C130" s="1" t="s">
         <v>304</v>
@@ -4751,7 +4769,7 @@
         <v>47</v>
       </c>
       <c r="E130" s="7" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="F130" s="1" t="n">
         <v>0</v>
@@ -4762,19 +4780,19 @@
     </row>
     <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A131" s="3" t="s">
+        <v>305</v>
+      </c>
+      <c r="B131" s="3" t="s">
+        <v>293</v>
+      </c>
+      <c r="C131" s="1" t="s">
         <v>306</v>
       </c>
-      <c r="B131" s="3" t="s">
-        <v>289</v>
-      </c>
-      <c r="C131" s="1" t="s">
-        <v>307</v>
-      </c>
       <c r="D131" s="1" t="s">
         <v>47</v>
       </c>
       <c r="E131" s="7" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="F131" s="1" t="n">
         <v>0</v>
@@ -4785,19 +4803,19 @@
     </row>
     <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A132" s="3" t="s">
+        <v>307</v>
+      </c>
+      <c r="B132" s="3" t="s">
+        <v>293</v>
+      </c>
+      <c r="C132" s="1" t="s">
         <v>308</v>
       </c>
-      <c r="B132" s="3" t="s">
-        <v>289</v>
-      </c>
-      <c r="C132" s="1" t="s">
+      <c r="D132" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E132" s="7" t="s">
         <v>309</v>
-      </c>
-      <c r="D132" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="E132" s="7" t="s">
-        <v>305</v>
       </c>
       <c r="F132" s="1" t="n">
         <v>0</v>
@@ -4811,7 +4829,7 @@
         <v>310</v>
       </c>
       <c r="B133" s="3" t="s">
-        <v>289</v>
+        <v>293</v>
       </c>
       <c r="C133" s="1" t="s">
         <v>311</v>
@@ -4820,7 +4838,7 @@
         <v>47</v>
       </c>
       <c r="E133" s="7" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
       <c r="F133" s="1" t="n">
         <v>0</v>
@@ -4831,19 +4849,19 @@
     </row>
     <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A134" s="3" t="s">
+        <v>312</v>
+      </c>
+      <c r="B134" s="3" t="s">
+        <v>293</v>
+      </c>
+      <c r="C134" s="1" t="s">
         <v>313</v>
       </c>
-      <c r="B134" s="3" t="s">
-        <v>289</v>
-      </c>
-      <c r="C134" s="1" t="s">
-        <v>314</v>
-      </c>
       <c r="D134" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="E134" s="1" t="s">
-        <v>315</v>
+      <c r="E134" s="7" t="s">
+        <v>309</v>
       </c>
       <c r="F134" s="1" t="n">
         <v>0</v>
@@ -4854,19 +4872,19 @@
     </row>
     <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A135" s="3" t="s">
+        <v>314</v>
+      </c>
+      <c r="B135" s="3" t="s">
+        <v>293</v>
+      </c>
+      <c r="C135" s="1" t="s">
+        <v>315</v>
+      </c>
+      <c r="D135" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E135" s="7" t="s">
         <v>316</v>
-      </c>
-      <c r="B135" s="3" t="s">
-        <v>289</v>
-      </c>
-      <c r="C135" s="1" t="s">
-        <v>317</v>
-      </c>
-      <c r="D135" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="E135" s="1" t="s">
-        <v>318</v>
       </c>
       <c r="F135" s="1" t="n">
         <v>0</v>
@@ -4877,19 +4895,19 @@
     </row>
     <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A136" s="3" t="s">
+        <v>317</v>
+      </c>
+      <c r="B136" s="3" t="s">
+        <v>293</v>
+      </c>
+      <c r="C136" s="1" t="s">
+        <v>318</v>
+      </c>
+      <c r="D136" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E136" s="1" t="s">
         <v>319</v>
-      </c>
-      <c r="B136" s="3" t="s">
-        <v>289</v>
-      </c>
-      <c r="C136" s="1" t="s">
-        <v>320</v>
-      </c>
-      <c r="D136" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="E136" s="1" t="s">
-        <v>321</v>
       </c>
       <c r="F136" s="1" t="n">
         <v>0</v>
@@ -4900,19 +4918,19 @@
     </row>
     <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A137" s="3" t="s">
+        <v>320</v>
+      </c>
+      <c r="B137" s="3" t="s">
+        <v>293</v>
+      </c>
+      <c r="C137" s="1" t="s">
+        <v>321</v>
+      </c>
+      <c r="D137" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E137" s="1" t="s">
         <v>322</v>
-      </c>
-      <c r="B137" s="3" t="s">
-        <v>289</v>
-      </c>
-      <c r="C137" s="1" t="s">
-        <v>323</v>
-      </c>
-      <c r="D137" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="E137" s="1" t="s">
-        <v>324</v>
       </c>
       <c r="F137" s="1" t="n">
         <v>0</v>
@@ -4923,19 +4941,19 @@
     </row>
     <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A138" s="3" t="s">
+        <v>323</v>
+      </c>
+      <c r="B138" s="3" t="s">
+        <v>293</v>
+      </c>
+      <c r="C138" s="1" t="s">
+        <v>324</v>
+      </c>
+      <c r="D138" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E138" s="1" t="s">
         <v>325</v>
-      </c>
-      <c r="B138" s="3" t="s">
-        <v>289</v>
-      </c>
-      <c r="C138" s="1" t="s">
-        <v>326</v>
-      </c>
-      <c r="D138" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="E138" s="1" t="s">
-        <v>327</v>
       </c>
       <c r="F138" s="1" t="n">
         <v>0</v>
@@ -4946,19 +4964,19 @@
     </row>
     <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A139" s="3" t="s">
+        <v>326</v>
+      </c>
+      <c r="B139" s="3" t="s">
+        <v>293</v>
+      </c>
+      <c r="C139" s="1" t="s">
+        <v>327</v>
+      </c>
+      <c r="D139" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E139" s="1" t="s">
         <v>328</v>
-      </c>
-      <c r="B139" s="3" t="s">
-        <v>289</v>
-      </c>
-      <c r="C139" s="1" t="s">
-        <v>329</v>
-      </c>
-      <c r="D139" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="E139" s="1" t="s">
-        <v>327</v>
       </c>
       <c r="F139" s="1" t="n">
         <v>0</v>
@@ -4969,28 +4987,25 @@
     </row>
     <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A140" s="3" t="s">
+        <v>329</v>
+      </c>
+      <c r="B140" s="3" t="s">
+        <v>293</v>
+      </c>
+      <c r="C140" s="1" t="s">
         <v>330</v>
       </c>
-      <c r="B140" s="3" t="s">
-        <v>289</v>
-      </c>
-      <c r="C140" s="1" t="s">
+      <c r="D140" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E140" s="1" t="s">
         <v>331</v>
       </c>
-      <c r="D140" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="E140" s="1" t="s">
-        <v>74</v>
-      </c>
       <c r="F140" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G140" s="1" t="n">
         <v>0</v>
-      </c>
-      <c r="H140" s="1" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4998,16 +5013,16 @@
         <v>332</v>
       </c>
       <c r="B141" s="3" t="s">
+        <v>293</v>
+      </c>
+      <c r="C141" s="1" t="s">
         <v>333</v>
       </c>
-      <c r="C141" s="1" t="s">
-        <v>334</v>
-      </c>
       <c r="D141" s="1" t="s">
         <v>47</v>
       </c>
       <c r="E141" s="1" t="s">
-        <v>335</v>
+        <v>331</v>
       </c>
       <c r="F141" s="1" t="n">
         <v>0</v>
@@ -5018,113 +5033,116 @@
     </row>
     <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A142" s="3" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="B142" s="3" t="s">
-        <v>333</v>
+        <v>293</v>
       </c>
       <c r="C142" s="1" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="D142" s="1" t="s">
         <v>47</v>
       </c>
       <c r="E142" s="1" t="s">
-        <v>338</v>
+        <v>74</v>
       </c>
       <c r="F142" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G142" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="H142" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A143" s="3" t="s">
+        <v>336</v>
+      </c>
+      <c r="B143" s="3" t="s">
+        <v>337</v>
+      </c>
+      <c r="C143" s="1" t="s">
+        <v>338</v>
+      </c>
+      <c r="D143" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E143" s="1" t="s">
         <v>339</v>
       </c>
-      <c r="B143" s="3" t="s">
-        <v>333</v>
-      </c>
-      <c r="C143" s="1" t="s">
-        <v>340</v>
-      </c>
-      <c r="D143" s="1" t="s">
-        <v>47</v>
-      </c>
       <c r="F143" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G143" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A144" s="3" t="s">
+        <v>340</v>
+      </c>
+      <c r="B144" s="3" t="s">
+        <v>337</v>
+      </c>
+      <c r="C144" s="1" t="s">
         <v>341</v>
       </c>
-      <c r="B144" s="3" t="s">
-        <v>333</v>
-      </c>
-      <c r="C144" s="1" t="s">
+      <c r="D144" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E144" s="1" t="s">
         <v>342</v>
       </c>
-      <c r="D144" s="1" t="s">
-        <v>47</v>
-      </c>
       <c r="F144" s="1" t="n">
         <v>0</v>
       </c>
+      <c r="G144" s="1" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A145" s="7" t="s">
+      <c r="A145" s="3" t="s">
         <v>343</v>
       </c>
-      <c r="B145" s="7" t="s">
+      <c r="B145" s="3" t="s">
+        <v>337</v>
+      </c>
+      <c r="C145" s="1" t="s">
         <v>344</v>
       </c>
-      <c r="C145" s="1" t="s">
+      <c r="D145" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="F145" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A146" s="3" t="s">
         <v>345</v>
       </c>
-      <c r="D145" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="E145" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="F145" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G145" s="1" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A146" s="7" t="s">
+      <c r="B146" s="3" t="s">
+        <v>337</v>
+      </c>
+      <c r="C146" s="1" t="s">
         <v>346</v>
       </c>
-      <c r="B146" s="7" t="s">
-        <v>344</v>
-      </c>
-      <c r="C146" s="1" t="s">
+      <c r="D146" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="F146" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A147" s="7" t="s">
         <v>347</v>
       </c>
-      <c r="D146" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="E146" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="F146" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G146" s="1" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A147" s="1" t="s">
+      <c r="B147" s="7" t="s">
         <v>348</v>
-      </c>
-      <c r="B147" s="7" t="s">
-        <v>344</v>
       </c>
       <c r="C147" s="1" t="s">
         <v>349</v>
@@ -5133,30 +5151,30 @@
         <v>47</v>
       </c>
       <c r="E147" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="F147" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G147" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A148" s="7" t="s">
         <v>350</v>
       </c>
-      <c r="F147" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G147" s="1" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A148" s="1" t="s">
+      <c r="B148" s="7" t="s">
+        <v>348</v>
+      </c>
+      <c r="C148" s="1" t="s">
         <v>351</v>
       </c>
-      <c r="B148" s="7" t="s">
-        <v>344</v>
-      </c>
-      <c r="C148" s="1" t="s">
-        <v>352</v>
-      </c>
       <c r="D148" s="1" t="s">
         <v>47</v>
       </c>
       <c r="E148" s="1" t="s">
-        <v>353</v>
+        <v>48</v>
       </c>
       <c r="F148" s="1" t="n">
         <v>0</v>
@@ -5167,19 +5185,19 @@
     </row>
     <row r="149" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A149" s="1" t="s">
+        <v>352</v>
+      </c>
+      <c r="B149" s="7" t="s">
+        <v>348</v>
+      </c>
+      <c r="C149" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="D149" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E149" s="1" t="s">
         <v>354</v>
-      </c>
-      <c r="B149" s="7" t="s">
-        <v>344</v>
-      </c>
-      <c r="C149" s="1" t="s">
-        <v>355</v>
-      </c>
-      <c r="D149" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="E149" s="1" t="s">
-        <v>356</v>
       </c>
       <c r="F149" s="1" t="n">
         <v>0</v>
@@ -5190,45 +5208,48 @@
     </row>
     <row r="150" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A150" s="1" t="s">
+        <v>355</v>
+      </c>
+      <c r="B150" s="7" t="s">
+        <v>348</v>
+      </c>
+      <c r="C150" s="1" t="s">
+        <v>356</v>
+      </c>
+      <c r="D150" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E150" s="1" t="s">
         <v>357</v>
       </c>
-      <c r="B150" s="7" t="s">
-        <v>344</v>
-      </c>
-      <c r="C150" s="1" t="s">
+      <c r="F150" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G150" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="151" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A151" s="1" t="s">
         <v>358</v>
       </c>
-      <c r="D150" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="F150" s="1" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="151" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A151" s="7" t="s">
+      <c r="B151" s="7" t="s">
+        <v>348</v>
+      </c>
+      <c r="C151" s="1" t="s">
         <v>359</v>
       </c>
-      <c r="B151" s="7" t="s">
-        <v>344</v>
-      </c>
-      <c r="C151" s="1" t="s">
+      <c r="D151" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E151" s="1" t="s">
         <v>360</v>
       </c>
-      <c r="D151" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="E151" s="1" t="s">
-        <v>74</v>
-      </c>
       <c r="F151" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G151" s="1" t="n">
         <v>0</v>
-      </c>
-      <c r="H151" s="1" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="152" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5236,7 +5257,7 @@
         <v>361</v>
       </c>
       <c r="B152" s="7" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
       <c r="C152" s="1" t="s">
         <v>362</v>
@@ -5244,19 +5265,16 @@
       <c r="D152" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="E152" s="1" t="s">
-        <v>104</v>
-      </c>
       <c r="F152" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="153" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A153" s="1" t="s">
+      <c r="A153" s="7" t="s">
         <v>363</v>
       </c>
       <c r="B153" s="7" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
       <c r="C153" s="1" t="s">
         <v>364</v>
@@ -5265,13 +5283,16 @@
         <v>47</v>
       </c>
       <c r="E153" s="1" t="s">
-        <v>195</v>
+        <v>74</v>
       </c>
       <c r="F153" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G153" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="H153" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="154" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5279,7 +5300,7 @@
         <v>365</v>
       </c>
       <c r="B154" s="7" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
       <c r="C154" s="1" t="s">
         <v>366</v>
@@ -5288,24 +5309,18 @@
         <v>47</v>
       </c>
       <c r="E154" s="1" t="s">
-        <v>154</v>
+        <v>106</v>
       </c>
       <c r="F154" s="1" t="n">
         <v>0</v>
-      </c>
-      <c r="G154" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H154" s="1" t="n">
-        <v>100</v>
       </c>
     </row>
     <row r="155" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A155" s="1" t="s">
         <v>367</v>
       </c>
-      <c r="B155" s="1" t="s">
-        <v>344</v>
+      <c r="B155" s="7" t="s">
+        <v>348</v>
       </c>
       <c r="C155" s="1" t="s">
         <v>368</v>
@@ -5314,7 +5329,7 @@
         <v>47</v>
       </c>
       <c r="E155" s="1" t="s">
-        <v>353</v>
+        <v>199</v>
       </c>
       <c r="F155" s="1" t="n">
         <v>0</v>
@@ -5327,8 +5342,8 @@
       <c r="A156" s="1" t="s">
         <v>369</v>
       </c>
-      <c r="B156" s="1" t="s">
-        <v>344</v>
+      <c r="B156" s="7" t="s">
+        <v>348</v>
       </c>
       <c r="C156" s="1" t="s">
         <v>370</v>
@@ -5337,21 +5352,24 @@
         <v>47</v>
       </c>
       <c r="E156" s="1" t="s">
-        <v>48</v>
+        <v>158</v>
       </c>
       <c r="F156" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G156" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="H156" s="1" t="n">
+        <v>100</v>
       </c>
     </row>
     <row r="157" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A157" s="1" t="s">
         <v>371</v>
       </c>
-      <c r="B157" s="7" t="s">
-        <v>344</v>
+      <c r="B157" s="1" t="s">
+        <v>348</v>
       </c>
       <c r="C157" s="1" t="s">
         <v>372</v>
@@ -5360,7 +5378,7 @@
         <v>47</v>
       </c>
       <c r="E157" s="1" t="s">
-        <v>48</v>
+        <v>357</v>
       </c>
       <c r="F157" s="1" t="n">
         <v>0</v>
@@ -5373,8 +5391,8 @@
       <c r="A158" s="1" t="s">
         <v>373</v>
       </c>
-      <c r="B158" s="7" t="s">
-        <v>344</v>
+      <c r="B158" s="1" t="s">
+        <v>348</v>
       </c>
       <c r="C158" s="1" t="s">
         <v>374</v>
@@ -5397,7 +5415,7 @@
         <v>375</v>
       </c>
       <c r="B159" s="7" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
       <c r="C159" s="1" t="s">
         <v>376</v>
@@ -5406,7 +5424,7 @@
         <v>47</v>
       </c>
       <c r="E159" s="1" t="s">
-        <v>377</v>
+        <v>48</v>
       </c>
       <c r="F159" s="1" t="n">
         <v>0</v>
@@ -5417,54 +5435,48 @@
     </row>
     <row r="160" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A160" s="1" t="s">
+        <v>377</v>
+      </c>
+      <c r="B160" s="7" t="s">
+        <v>348</v>
+      </c>
+      <c r="C160" s="1" t="s">
         <v>378</v>
       </c>
-      <c r="B160" s="7" t="s">
-        <v>344</v>
-      </c>
-      <c r="C160" s="1" t="s">
-        <v>379</v>
-      </c>
       <c r="D160" s="1" t="s">
         <v>47</v>
       </c>
       <c r="E160" s="1" t="s">
-        <v>154</v>
+        <v>48</v>
       </c>
       <c r="F160" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G160" s="1" t="n">
         <v>0</v>
-      </c>
-      <c r="H160" s="1" t="n">
-        <v>100</v>
       </c>
     </row>
     <row r="161" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A161" s="1" t="s">
+        <v>379</v>
+      </c>
+      <c r="B161" s="7" t="s">
+        <v>348</v>
+      </c>
+      <c r="C161" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="B161" s="7" t="s">
-        <v>344</v>
-      </c>
-      <c r="C161" s="1" t="s">
+      <c r="D161" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E161" s="1" t="s">
         <v>381</v>
       </c>
-      <c r="D161" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="E161" s="1" t="s">
-        <v>74</v>
-      </c>
       <c r="F161" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G161" s="1" t="n">
         <v>0</v>
-      </c>
-      <c r="H161" s="1" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="162" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5472,16 +5484,16 @@
         <v>382</v>
       </c>
       <c r="B162" s="7" t="s">
-        <v>344</v>
-      </c>
-      <c r="C162" s="7" t="s">
+        <v>348</v>
+      </c>
+      <c r="C162" s="1" t="s">
         <v>383</v>
       </c>
       <c r="D162" s="1" t="s">
         <v>47</v>
       </c>
       <c r="E162" s="1" t="s">
-        <v>74</v>
+        <v>158</v>
       </c>
       <c r="F162" s="1" t="n">
         <v>0</v>
@@ -5490,7 +5502,7 @@
         <v>0</v>
       </c>
       <c r="H162" s="1" t="n">
-        <v>1</v>
+        <v>100</v>
       </c>
     </row>
     <row r="163" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5498,9 +5510,9 @@
         <v>384</v>
       </c>
       <c r="B163" s="7" t="s">
-        <v>344</v>
-      </c>
-      <c r="C163" s="7" t="s">
+        <v>348</v>
+      </c>
+      <c r="C163" s="1" t="s">
         <v>385</v>
       </c>
       <c r="D163" s="1" t="s">
@@ -5524,22 +5536,25 @@
         <v>386</v>
       </c>
       <c r="B164" s="7" t="s">
-        <v>344</v>
-      </c>
-      <c r="C164" s="1" t="s">
+        <v>348</v>
+      </c>
+      <c r="C164" s="7" t="s">
         <v>387</v>
       </c>
       <c r="D164" s="1" t="s">
         <v>47</v>
       </c>
       <c r="E164" s="1" t="s">
-        <v>377</v>
+        <v>74</v>
       </c>
       <c r="F164" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G164" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="H164" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="165" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5547,25 +5562,73 @@
         <v>388</v>
       </c>
       <c r="B165" s="7" t="s">
-        <v>344</v>
-      </c>
-      <c r="C165" s="1" t="s">
+        <v>348</v>
+      </c>
+      <c r="C165" s="7" t="s">
         <v>389</v>
       </c>
       <c r="D165" s="1" t="s">
         <v>47</v>
       </c>
       <c r="E165" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="F165" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G165" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H165" s="1" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="166" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A166" s="1" t="s">
+        <v>390</v>
+      </c>
+      <c r="B166" s="7" t="s">
+        <v>348</v>
+      </c>
+      <c r="C166" s="1" t="s">
+        <v>391</v>
+      </c>
+      <c r="D166" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E166" s="1" t="s">
+        <v>381</v>
+      </c>
+      <c r="F166" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G166" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="167" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A167" s="1" t="s">
+        <v>392</v>
+      </c>
+      <c r="B167" s="7" t="s">
+        <v>348</v>
+      </c>
+      <c r="C167" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="D167" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E167" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="F165" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G165" s="1" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+      <c r="F167" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G167" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
defoliation params in SpParams
</commit_message>
<xml_diff>
--- a/data-raw/SpParamsDefinition.xlsx
+++ b/data-raw/SpParamsDefinition.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="true"/>
   <workbookProtection/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="814" uniqueCount="400">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="829" uniqueCount="406">
   <si>
     <t xml:space="preserve">ParameterName</t>
   </si>
@@ -409,6 +409,27 @@
     <t xml:space="preserve">Degree days corresponding to leaf fall</t>
   </si>
   <si>
+    <t xml:space="preserve">LeafPLCCrit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Critical proportion loss of conductance associated with cavitation-induced leaf senescence</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[0,1]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BudPLCCrit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Critical proportion loss of conductance associated with cavitation-induced bud (branch) senescence</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LeafTSCrit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Critical temperature associated to heat-induced leaf senescence</t>
+  </si>
+  <si>
     <t xml:space="preserve">SLA</t>
   </si>
   <si>
@@ -446,9 +467,6 @@
   </si>
   <si>
     <t xml:space="preserve">Proportion of sapwood corresponding to conducive elements (vessels or tracheids) as opposed to parenchymatic tissue.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[0,1]</t>
   </si>
   <si>
     <t xml:space="preserve">r635</t>
@@ -1882,37 +1900,37 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="000000"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="18a303"/>
+        <a:srgbClr val="18A303"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="0369a3"/>
+        <a:srgbClr val="0369A3"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="a33e03"/>
+        <a:srgbClr val="A33E03"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8e03a3"/>
+        <a:srgbClr val="8E03A3"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="c99c00"/>
+        <a:srgbClr val="C99C00"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="c9211e"/>
+        <a:srgbClr val="C9211E"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ee"/>
+        <a:srgbClr val="0000EE"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="551a8b"/>
+        <a:srgbClr val="551A8B"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
@@ -1985,10 +2003,10 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H170"/>
-  <sheetFormatPr defaultColWidth="10.25" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:H173"/>
+  <sheetFormatPr defaultColWidth="10.2578125" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="25.25"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="35.53"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="26.26"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="48.2"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="11.32"/>
@@ -3154,85 +3172,88 @@
         <v>129</v>
       </c>
       <c r="B59" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="C59" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="C59" s="1" t="s">
+      <c r="D59" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E59" s="5" t="s">
         <v>131</v>
       </c>
-      <c r="D59" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="E59" s="5" t="s">
+      <c r="F59" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G59" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H59" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="F59" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G59" s="1" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="3" t="s">
+      <c r="B60" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="C60" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="B60" s="6" t="s">
-        <v>130</v>
-      </c>
-      <c r="C60" s="1" t="s">
+      <c r="D60" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E60" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="F60" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G60" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H60" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="D60" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="E60" s="1" t="s">
+      <c r="B61" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="C61" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="F60" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G60" s="1" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="3" t="s">
+      <c r="D61" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E61" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="F61" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="B61" s="6" t="s">
-        <v>130</v>
-      </c>
-      <c r="C61" s="1" t="s">
+      <c r="B62" s="6" t="s">
         <v>137</v>
       </c>
-      <c r="D61" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="E61" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="F61" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G61" s="1" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="3" t="s">
+      <c r="C62" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="B62" s="6" t="s">
-        <v>130</v>
-      </c>
-      <c r="C62" s="1" t="s">
+      <c r="D62" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E62" s="5" t="s">
         <v>139</v>
-      </c>
-      <c r="D62" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="E62" s="1" t="s">
-        <v>135</v>
       </c>
       <c r="F62" s="1" t="n">
         <v>0</v>
@@ -3246,7 +3267,7 @@
         <v>140</v>
       </c>
       <c r="B63" s="6" t="s">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="C63" s="1" t="s">
         <v>141</v>
@@ -3262,9 +3283,6 @@
       </c>
       <c r="G63" s="1" t="n">
         <v>0</v>
-      </c>
-      <c r="H63" s="1" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3272,7 +3290,7 @@
         <v>143</v>
       </c>
       <c r="B64" s="6" t="s">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="C64" s="1" t="s">
         <v>144</v>
@@ -3280,30 +3298,30 @@
       <c r="D64" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="E64" s="5" t="s">
-        <v>145</v>
+      <c r="E64" s="1" t="s">
+        <v>142</v>
       </c>
       <c r="F64" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G64" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="B65" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="C65" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="B65" s="6" t="s">
-        <v>130</v>
-      </c>
-      <c r="C65" s="1" t="s">
-        <v>147</v>
-      </c>
       <c r="D65" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="E65" s="5" t="s">
+      <c r="E65" s="1" t="s">
         <v>142</v>
       </c>
       <c r="F65" s="1" t="n">
@@ -3311,95 +3329,98 @@
       </c>
       <c r="G65" s="1" t="n">
         <v>0</v>
-      </c>
-      <c r="H65" s="1" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="B66" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="C66" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="B66" s="6" t="s">
-        <v>130</v>
-      </c>
-      <c r="C66" s="1" t="s">
-        <v>149</v>
-      </c>
       <c r="D66" s="1" t="s">
         <v>51</v>
       </c>
       <c r="E66" s="1" t="s">
-        <v>150</v>
+        <v>131</v>
       </c>
       <c r="F66" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G66" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="H66" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="B67" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="C67" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="D67" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E67" s="5" t="s">
         <v>151</v>
       </c>
-      <c r="B67" s="6" t="s">
-        <v>130</v>
-      </c>
-      <c r="C67" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="D67" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="E67" s="7" t="s">
-        <v>150</v>
-      </c>
       <c r="F67" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G67" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="B68" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="C68" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="B68" s="6" t="s">
-        <v>130</v>
-      </c>
-      <c r="C68" s="1" t="s">
-        <v>154</v>
-      </c>
       <c r="D68" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="E68" s="1" t="s">
-        <v>52</v>
+      <c r="E68" s="5" t="s">
+        <v>131</v>
       </c>
       <c r="F68" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G68" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="H68" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="B69" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="C69" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="B69" s="6" t="s">
-        <v>130</v>
-      </c>
-      <c r="C69" s="1" t="s">
+      <c r="D69" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E69" s="1" t="s">
         <v>156</v>
-      </c>
-      <c r="D69" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="E69" s="1" t="s">
-        <v>157</v>
       </c>
       <c r="F69" s="1" t="n">
         <v>0</v>
@@ -3410,19 +3431,19 @@
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="B70" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="C70" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="B70" s="6" t="s">
-        <v>130</v>
-      </c>
-      <c r="C70" s="1" t="s">
-        <v>159</v>
-      </c>
       <c r="D70" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="E70" s="1" t="s">
-        <v>160</v>
+      <c r="E70" s="7" t="s">
+        <v>156</v>
       </c>
       <c r="F70" s="1" t="n">
         <v>0</v>
@@ -3433,19 +3454,19 @@
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="3" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="B71" s="6" t="s">
-        <v>162</v>
+        <v>137</v>
       </c>
       <c r="C71" s="1" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="D71" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="E71" s="5" t="s">
-        <v>164</v>
+      <c r="E71" s="1" t="s">
+        <v>52</v>
       </c>
       <c r="F71" s="1" t="n">
         <v>0</v>
@@ -3456,19 +3477,19 @@
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="3" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="B72" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="C72" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="C72" s="1" t="s">
-        <v>166</v>
-      </c>
       <c r="D72" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="E72" s="5" t="s">
-        <v>164</v>
+      <c r="E72" s="1" t="s">
+        <v>163</v>
       </c>
       <c r="F72" s="1" t="n">
         <v>0</v>
@@ -3479,65 +3500,65 @@
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="3" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="B73" s="6" t="s">
-        <v>162</v>
+        <v>137</v>
       </c>
       <c r="C73" s="1" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="D73" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="E73" s="5" t="s">
-        <v>169</v>
+      <c r="E73" s="1" t="s">
+        <v>166</v>
       </c>
       <c r="F73" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="H73" s="1" t="n">
+      <c r="G73" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="B74" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="C74" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="D74" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E74" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="B74" s="6" t="s">
-        <v>162</v>
-      </c>
-      <c r="C74" s="1" t="s">
-        <v>171</v>
-      </c>
-      <c r="D74" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="E74" s="5" t="s">
-        <v>169</v>
-      </c>
       <c r="F74" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="H74" s="1" t="n">
+      <c r="G74" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="B75" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="C75" s="1" t="s">
         <v>172</v>
       </c>
-      <c r="B75" s="6" t="s">
-        <v>162</v>
-      </c>
-      <c r="C75" s="1" t="s">
-        <v>173</v>
-      </c>
       <c r="D75" s="1" t="s">
         <v>51</v>
       </c>
       <c r="E75" s="5" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="F75" s="1" t="n">
         <v>0</v>
@@ -3548,28 +3569,25 @@
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="B76" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="C76" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="B76" s="6" t="s">
-        <v>162</v>
-      </c>
-      <c r="C76" s="1" t="s">
+      <c r="D76" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E76" s="5" t="s">
         <v>175</v>
       </c>
-      <c r="D76" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="E76" s="5" t="s">
-        <v>142</v>
-      </c>
       <c r="F76" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="G76" s="1" t="n">
-        <v>0</v>
-      </c>
       <c r="H76" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3577,7 +3595,7 @@
         <v>176</v>
       </c>
       <c r="B77" s="6" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
       <c r="C77" s="1" t="s">
         <v>177</v>
@@ -3586,7 +3604,7 @@
         <v>51</v>
       </c>
       <c r="E77" s="5" t="s">
-        <v>169</v>
+        <v>175</v>
       </c>
       <c r="F77" s="1" t="n">
         <v>0</v>
@@ -3600,7 +3618,7 @@
         <v>178</v>
       </c>
       <c r="B78" s="6" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
       <c r="C78" s="1" t="s">
         <v>179</v>
@@ -3609,7 +3627,7 @@
         <v>51</v>
       </c>
       <c r="E78" s="5" t="s">
-        <v>169</v>
+        <v>175</v>
       </c>
       <c r="F78" s="1" t="n">
         <v>0</v>
@@ -3623,7 +3641,7 @@
         <v>180</v>
       </c>
       <c r="B79" s="6" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
       <c r="C79" s="1" t="s">
         <v>181</v>
@@ -3632,7 +3650,7 @@
         <v>51</v>
       </c>
       <c r="E79" s="5" t="s">
-        <v>142</v>
+        <v>131</v>
       </c>
       <c r="F79" s="1" t="n">
         <v>0</v>
@@ -3649,39 +3667,39 @@
         <v>182</v>
       </c>
       <c r="B80" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="C80" s="1" t="s">
         <v>183</v>
       </c>
-      <c r="C80" s="1" t="s">
-        <v>184</v>
-      </c>
       <c r="D80" s="1" t="s">
         <v>51</v>
       </c>
       <c r="E80" s="5" t="s">
-        <v>185</v>
+        <v>175</v>
       </c>
       <c r="F80" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="G80" s="1" t="n">
+      <c r="H80" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="3" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="B81" s="6" t="s">
-        <v>183</v>
+        <v>168</v>
       </c>
       <c r="C81" s="1" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="D81" s="1" t="s">
         <v>51</v>
       </c>
       <c r="E81" s="5" t="s">
-        <v>188</v>
+        <v>175</v>
       </c>
       <c r="F81" s="1" t="n">
         <v>0</v>
@@ -3692,42 +3710,45 @@
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="3" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="B82" s="6" t="s">
-        <v>183</v>
+        <v>168</v>
       </c>
       <c r="C82" s="1" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="D82" s="1" t="s">
         <v>51</v>
       </c>
       <c r="E82" s="5" t="s">
-        <v>164</v>
+        <v>131</v>
       </c>
       <c r="F82" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G82" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="H82" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="B83" s="6" t="s">
+        <v>189</v>
+      </c>
+      <c r="C83" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="D83" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E83" s="5" t="s">
         <v>191</v>
-      </c>
-      <c r="B83" s="6" t="s">
-        <v>183</v>
-      </c>
-      <c r="C83" s="1" t="s">
-        <v>192</v>
-      </c>
-      <c r="D83" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="E83" s="5" t="s">
-        <v>164</v>
       </c>
       <c r="F83" s="1" t="n">
         <v>0</v>
@@ -3738,19 +3759,19 @@
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="B84" s="6" t="s">
+        <v>189</v>
+      </c>
+      <c r="C84" s="1" t="s">
         <v>193</v>
       </c>
-      <c r="B84" s="6" t="s">
-        <v>183</v>
-      </c>
-      <c r="C84" s="1" t="s">
+      <c r="D84" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E84" s="5" t="s">
         <v>194</v>
-      </c>
-      <c r="D84" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="E84" s="5" t="s">
-        <v>164</v>
       </c>
       <c r="F84" s="1" t="n">
         <v>0</v>
@@ -3764,42 +3785,39 @@
         <v>195</v>
       </c>
       <c r="B85" s="6" t="s">
+        <v>189</v>
+      </c>
+      <c r="C85" s="1" t="s">
         <v>196</v>
       </c>
-      <c r="C85" s="1" t="s">
-        <v>197</v>
-      </c>
       <c r="D85" s="1" t="s">
         <v>51</v>
       </c>
       <c r="E85" s="5" t="s">
-        <v>198</v>
+        <v>170</v>
       </c>
       <c r="F85" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G85" s="1" t="n">
         <v>0</v>
-      </c>
-      <c r="H85" s="1" t="n">
-        <v>90</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="3" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="B86" s="6" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
       <c r="C86" s="1" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="D86" s="1" t="s">
         <v>51</v>
       </c>
       <c r="E86" s="5" t="s">
-        <v>198</v>
+        <v>170</v>
       </c>
       <c r="F86" s="1" t="n">
         <v>0</v>
@@ -3810,19 +3828,19 @@
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="3" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="B87" s="6" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
       <c r="C87" s="1" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="D87" s="1" t="s">
         <v>51</v>
       </c>
       <c r="E87" s="5" t="s">
-        <v>78</v>
+        <v>170</v>
       </c>
       <c r="F87" s="1" t="n">
         <v>0</v>
@@ -3833,42 +3851,45 @@
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="B88" s="6" t="s">
+        <v>202</v>
+      </c>
+      <c r="C88" s="1" t="s">
         <v>203</v>
       </c>
-      <c r="B88" s="6" t="s">
-        <v>196</v>
-      </c>
-      <c r="C88" s="1" t="s">
+      <c r="D88" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E88" s="5" t="s">
         <v>204</v>
       </c>
-      <c r="D88" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="E88" s="5" t="s">
-        <v>205</v>
-      </c>
       <c r="F88" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G88" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="H88" s="1" t="n">
+        <v>90</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="3" t="s">
+        <v>205</v>
+      </c>
+      <c r="B89" s="6" t="s">
+        <v>202</v>
+      </c>
+      <c r="C89" s="1" t="s">
         <v>206</v>
       </c>
-      <c r="B89" s="6" t="s">
-        <v>196</v>
-      </c>
-      <c r="C89" s="1" t="s">
-        <v>207</v>
-      </c>
       <c r="D89" s="1" t="s">
         <v>51</v>
       </c>
       <c r="E89" s="5" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="F89" s="1" t="n">
         <v>0</v>
@@ -3879,19 +3900,19 @@
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="3" t="s">
+        <v>207</v>
+      </c>
+      <c r="B90" s="6" t="s">
+        <v>202</v>
+      </c>
+      <c r="C90" s="1" t="s">
         <v>208</v>
       </c>
-      <c r="B90" s="6" t="s">
-        <v>196</v>
-      </c>
-      <c r="C90" s="1" t="s">
-        <v>209</v>
-      </c>
       <c r="D90" s="1" t="s">
         <v>51</v>
       </c>
       <c r="E90" s="5" t="s">
-        <v>205</v>
+        <v>78</v>
       </c>
       <c r="F90" s="1" t="n">
         <v>0</v>
@@ -3902,19 +3923,19 @@
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="3" t="s">
+        <v>209</v>
+      </c>
+      <c r="B91" s="6" t="s">
+        <v>202</v>
+      </c>
+      <c r="C91" s="1" t="s">
         <v>210</v>
       </c>
-      <c r="B91" s="6" t="s">
-        <v>196</v>
-      </c>
-      <c r="C91" s="1" t="s">
+      <c r="D91" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E91" s="5" t="s">
         <v>211</v>
-      </c>
-      <c r="D91" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="E91" s="5" t="s">
-        <v>212</v>
       </c>
       <c r="F91" s="1" t="n">
         <v>0</v>
@@ -3925,72 +3946,82 @@
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="3" t="s">
+        <v>212</v>
+      </c>
+      <c r="B92" s="6" t="s">
+        <v>202</v>
+      </c>
+      <c r="C92" s="1" t="s">
         <v>213</v>
       </c>
-      <c r="B92" s="6" t="s">
-        <v>214</v>
-      </c>
-      <c r="C92" s="1" t="s">
-        <v>215</v>
-      </c>
       <c r="D92" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="E92" s="5"/>
+      <c r="E92" s="5" t="s">
+        <v>211</v>
+      </c>
       <c r="F92" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G92" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="3" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="B93" s="6" t="s">
-        <v>214</v>
+        <v>202</v>
       </c>
       <c r="C93" s="1" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="D93" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="E93" s="5"/>
+      <c r="E93" s="5" t="s">
+        <v>211</v>
+      </c>
       <c r="F93" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G93" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="3" t="s">
+        <v>216</v>
+      </c>
+      <c r="B94" s="6" t="s">
+        <v>202</v>
+      </c>
+      <c r="C94" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="D94" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E94" s="5" t="s">
         <v>218</v>
       </c>
-      <c r="B94" s="6" t="s">
-        <v>214</v>
-      </c>
-      <c r="C94" s="1" t="s">
-        <v>219</v>
-      </c>
-      <c r="D94" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="E94" s="5" t="s">
-        <v>220</v>
-      </c>
       <c r="F94" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="H94" s="1" t="n">
+      <c r="G94" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="B95" s="6" t="s">
+        <v>220</v>
+      </c>
+      <c r="C95" s="1" t="s">
         <v>221</v>
-      </c>
-      <c r="B95" s="6" t="s">
-        <v>214</v>
-      </c>
-      <c r="C95" s="1" t="s">
-        <v>222</v>
       </c>
       <c r="D95" s="1" t="s">
         <v>51</v>
@@ -3999,60 +4030,57 @@
       <c r="F95" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="G95" s="1" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="3" t="s">
+        <v>222</v>
+      </c>
+      <c r="B96" s="6" t="s">
+        <v>220</v>
+      </c>
+      <c r="C96" s="1" t="s">
         <v>223</v>
       </c>
-      <c r="B96" s="6" t="s">
-        <v>214</v>
-      </c>
-      <c r="C96" s="1" t="s">
-        <v>224</v>
-      </c>
       <c r="D96" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="E96" s="5" t="s">
-        <v>225</v>
-      </c>
+      <c r="E96" s="5"/>
       <c r="F96" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G96" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="3" t="s">
+        <v>224</v>
+      </c>
+      <c r="B97" s="6" t="s">
+        <v>220</v>
+      </c>
+      <c r="C97" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="D97" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E97" s="5" t="s">
         <v>226</v>
       </c>
-      <c r="B97" s="6" t="s">
-        <v>214</v>
-      </c>
-      <c r="C97" s="1" t="s">
-        <v>227</v>
-      </c>
-      <c r="D97" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="E97" s="5"/>
       <c r="F97" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H97" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="B98" s="6" t="s">
+        <v>220</v>
+      </c>
+      <c r="C98" s="1" t="s">
         <v>228</v>
-      </c>
-      <c r="B98" s="6" t="s">
-        <v>214</v>
-      </c>
-      <c r="C98" s="1" t="s">
-        <v>229</v>
       </c>
       <c r="D98" s="1" t="s">
         <v>51</v>
@@ -4061,115 +4089,116 @@
       <c r="F98" s="1" t="n">
         <v>0</v>
       </c>
+      <c r="G98" s="1" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="B99" s="6" t="s">
+        <v>220</v>
+      </c>
+      <c r="C99" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="B99" s="6" t="s">
-        <v>214</v>
-      </c>
-      <c r="C99" s="1" t="s">
+      <c r="D99" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E99" s="5" t="s">
         <v>231</v>
       </c>
-      <c r="D99" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="E99" s="5"/>
       <c r="F99" s="1" t="n">
         <v>0</v>
       </c>
-    </row>
-    <row r="100" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G99" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="3" t="s">
         <v>232</v>
       </c>
       <c r="B100" s="6" t="s">
-        <v>214</v>
-      </c>
-      <c r="C100" s="8" t="s">
+        <v>220</v>
+      </c>
+      <c r="C100" s="1" t="s">
         <v>233</v>
       </c>
       <c r="D100" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="E100" s="5" t="s">
-        <v>234</v>
-      </c>
+      <c r="E100" s="5"/>
       <c r="F100" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G100" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="3" t="s">
+        <v>234</v>
+      </c>
+      <c r="B101" s="6" t="s">
+        <v>220</v>
+      </c>
+      <c r="C101" s="1" t="s">
         <v>235</v>
       </c>
-      <c r="B101" s="6" t="s">
-        <v>214</v>
-      </c>
-      <c r="C101" s="1" t="s">
-        <v>236</v>
-      </c>
       <c r="D101" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="E101" s="5" t="s">
-        <v>234</v>
-      </c>
+      <c r="E101" s="5"/>
       <c r="F101" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G101" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="3" t="s">
+        <v>236</v>
+      </c>
+      <c r="B102" s="6" t="s">
+        <v>220</v>
+      </c>
+      <c r="C102" s="1" t="s">
         <v>237</v>
       </c>
-      <c r="B102" s="6" t="s">
-        <v>214</v>
-      </c>
-      <c r="C102" s="1" t="s">
+      <c r="D102" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E102" s="5"/>
+      <c r="F102" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="103" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A103" s="3" t="s">
         <v>238</v>
       </c>
-      <c r="D102" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="E102" s="5" t="s">
-        <v>110</v>
-      </c>
-      <c r="F102" s="1" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="103" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A103" s="3" t="s">
+      <c r="B103" s="6" t="s">
+        <v>220</v>
+      </c>
+      <c r="C103" s="8" t="s">
         <v>239</v>
       </c>
-      <c r="B103" s="6" t="s">
-        <v>214</v>
-      </c>
-      <c r="C103" s="1" t="s">
+      <c r="D103" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E103" s="5" t="s">
         <v>240</v>
       </c>
-      <c r="D103" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="E103" s="5"/>
       <c r="F103" s="1" t="n">
         <v>0</v>
       </c>
-    </row>
-    <row r="104" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G103" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="3" t="s">
         <v>241</v>
       </c>
       <c r="B104" s="6" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="C104" s="1" t="s">
         <v>242</v>
@@ -4178,100 +4207,91 @@
         <v>51</v>
       </c>
       <c r="E104" s="5" t="s">
+        <v>240</v>
+      </c>
+      <c r="F104" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G104" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A105" s="3" t="s">
         <v>243</v>
       </c>
-      <c r="F104" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G104" s="1" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="105" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A105" s="3" t="s">
+      <c r="B105" s="6" t="s">
+        <v>220</v>
+      </c>
+      <c r="C105" s="1" t="s">
         <v>244</v>
       </c>
-      <c r="B105" s="6" t="s">
-        <v>214</v>
-      </c>
-      <c r="C105" s="1" t="s">
-        <v>245</v>
-      </c>
       <c r="D105" s="1" t="s">
         <v>51</v>
       </c>
       <c r="E105" s="5" t="s">
-        <v>220</v>
+        <v>110</v>
       </c>
       <c r="F105" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H105" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="3" t="s">
+        <v>245</v>
+      </c>
+      <c r="B106" s="6" t="s">
+        <v>220</v>
+      </c>
+      <c r="C106" s="1" t="s">
         <v>246</v>
       </c>
-      <c r="B106" s="6" t="s">
-        <v>214</v>
-      </c>
-      <c r="C106" s="1" t="s">
-        <v>247</v>
-      </c>
       <c r="D106" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="E106" s="5" t="s">
-        <v>248</v>
-      </c>
+      <c r="E106" s="5"/>
       <c r="F106" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="G106" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H106" s="1"/>
     </row>
     <row r="107" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="B107" s="6" t="s">
+        <v>220</v>
+      </c>
+      <c r="C107" s="1" t="s">
+        <v>248</v>
+      </c>
+      <c r="D107" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E107" s="5" t="s">
         <v>249</v>
       </c>
-      <c r="B107" s="6" t="s">
-        <v>214</v>
-      </c>
-      <c r="C107" s="1" t="s">
+      <c r="F107" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G107" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="108" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A108" s="3" t="s">
         <v>250</v>
       </c>
-      <c r="D107" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="E107" s="5" t="s">
+      <c r="B108" s="6" t="s">
+        <v>220</v>
+      </c>
+      <c r="C108" s="1" t="s">
         <v>251</v>
       </c>
-      <c r="F107" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G107" s="1" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A108" s="3" t="s">
-        <v>252</v>
-      </c>
-      <c r="B108" s="6" t="s">
-        <v>214</v>
-      </c>
-      <c r="C108" s="1" t="s">
-        <v>253</v>
-      </c>
       <c r="D108" s="1" t="s">
         <v>51</v>
       </c>
       <c r="E108" s="5" t="s">
-        <v>220</v>
+        <v>226</v>
       </c>
       <c r="F108" s="1" t="n">
         <v>0</v>
@@ -4282,47 +4302,48 @@
     </row>
     <row r="109" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="3" t="s">
+        <v>252</v>
+      </c>
+      <c r="B109" s="6" t="s">
+        <v>220</v>
+      </c>
+      <c r="C109" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="D109" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E109" s="5" t="s">
         <v>254</v>
       </c>
-      <c r="B109" s="6" t="s">
-        <v>214</v>
-      </c>
-      <c r="C109" s="1" t="s">
-        <v>255</v>
-      </c>
-      <c r="D109" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="E109" s="5" t="s">
-        <v>220</v>
-      </c>
       <c r="F109" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="H109" s="1" t="n">
-        <v>0</v>
-      </c>
+      <c r="G109" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H109" s="1"/>
     </row>
     <row r="110" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="3" t="s">
+        <v>255</v>
+      </c>
+      <c r="B110" s="6" t="s">
+        <v>220</v>
+      </c>
+      <c r="C110" s="1" t="s">
         <v>256</v>
       </c>
-      <c r="B110" s="6" t="s">
-        <v>214</v>
-      </c>
-      <c r="C110" s="1" t="s">
+      <c r="D110" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E110" s="5" t="s">
         <v>257</v>
       </c>
-      <c r="D110" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="E110" s="5" t="s">
-        <v>220</v>
-      </c>
       <c r="F110" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="H110" s="1" t="n">
+      <c r="G110" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4331,7 +4352,7 @@
         <v>258</v>
       </c>
       <c r="B111" s="6" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="C111" s="1" t="s">
         <v>259</v>
@@ -4340,22 +4361,21 @@
         <v>51</v>
       </c>
       <c r="E111" s="5" t="s">
-        <v>248</v>
+        <v>226</v>
       </c>
       <c r="F111" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="G111" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H111" s="1"/>
-    </row>
-    <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="H111" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="112" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="3" t="s">
         <v>260</v>
       </c>
       <c r="B112" s="6" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="C112" s="1" t="s">
         <v>261</v>
@@ -4364,7 +4384,7 @@
         <v>51</v>
       </c>
       <c r="E112" s="5" t="s">
-        <v>220</v>
+        <v>226</v>
       </c>
       <c r="F112" s="1" t="n">
         <v>0</v>
@@ -4378,7 +4398,7 @@
         <v>262</v>
       </c>
       <c r="B113" s="6" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="C113" s="1" t="s">
         <v>263</v>
@@ -4387,7 +4407,7 @@
         <v>51</v>
       </c>
       <c r="E113" s="5" t="s">
-        <v>220</v>
+        <v>226</v>
       </c>
       <c r="F113" s="1" t="n">
         <v>0</v>
@@ -4396,12 +4416,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="114" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="3" t="s">
         <v>264</v>
       </c>
       <c r="B114" s="6" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="C114" s="1" t="s">
         <v>265</v>
@@ -4410,21 +4430,22 @@
         <v>51</v>
       </c>
       <c r="E114" s="5" t="s">
-        <v>220</v>
+        <v>254</v>
       </c>
       <c r="F114" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="H114" s="1" t="n">
-        <v>0</v>
-      </c>
+      <c r="G114" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H114" s="1"/>
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A115" s="3" t="s">
         <v>266</v>
       </c>
       <c r="B115" s="6" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="C115" s="1" t="s">
         <v>267</v>
@@ -4433,22 +4454,21 @@
         <v>51</v>
       </c>
       <c r="E115" s="5" t="s">
-        <v>248</v>
+        <v>226</v>
       </c>
       <c r="F115" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="G115" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H115" s="1"/>
-    </row>
-    <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="H115" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="116" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A116" s="3" t="s">
         <v>268</v>
       </c>
       <c r="B116" s="6" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="C116" s="1" t="s">
         <v>269</v>
@@ -4457,30 +4477,30 @@
         <v>51</v>
       </c>
       <c r="E116" s="5" t="s">
+        <v>226</v>
+      </c>
+      <c r="F116" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H116" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="117" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A117" s="3" t="s">
         <v>270</v>
       </c>
-      <c r="F116" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G116" s="1" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A117" s="3" t="s">
+      <c r="B117" s="6" t="s">
+        <v>220</v>
+      </c>
+      <c r="C117" s="1" t="s">
         <v>271</v>
       </c>
-      <c r="B117" s="6" t="s">
-        <v>214</v>
-      </c>
-      <c r="C117" s="1" t="s">
-        <v>272</v>
-      </c>
       <c r="D117" s="1" t="s">
         <v>51</v>
       </c>
       <c r="E117" s="5" t="s">
-        <v>220</v>
+        <v>226</v>
       </c>
       <c r="F117" s="1" t="n">
         <v>0</v>
@@ -4491,47 +4511,48 @@
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A118" s="3" t="s">
+        <v>272</v>
+      </c>
+      <c r="B118" s="6" t="s">
+        <v>220</v>
+      </c>
+      <c r="C118" s="1" t="s">
         <v>273</v>
       </c>
-      <c r="B118" s="6" t="s">
-        <v>214</v>
-      </c>
-      <c r="C118" s="1" t="s">
-        <v>274</v>
-      </c>
       <c r="D118" s="1" t="s">
         <v>51</v>
       </c>
       <c r="E118" s="5" t="s">
-        <v>220</v>
+        <v>254</v>
       </c>
       <c r="F118" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="H118" s="1" t="n">
-        <v>0</v>
-      </c>
+      <c r="G118" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H118" s="1"/>
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A119" s="3" t="s">
+        <v>274</v>
+      </c>
+      <c r="B119" s="6" t="s">
+        <v>220</v>
+      </c>
+      <c r="C119" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="B119" s="6" t="s">
-        <v>214</v>
-      </c>
-      <c r="C119" s="1" t="s">
+      <c r="D119" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E119" s="5" t="s">
         <v>276</v>
       </c>
-      <c r="D119" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="E119" s="5" t="s">
-        <v>220</v>
-      </c>
       <c r="F119" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="H119" s="1" t="n">
+      <c r="G119" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4540,7 +4561,7 @@
         <v>277</v>
       </c>
       <c r="B120" s="6" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="C120" s="1" t="s">
         <v>278</v>
@@ -4549,22 +4570,21 @@
         <v>51</v>
       </c>
       <c r="E120" s="5" t="s">
-        <v>248</v>
+        <v>226</v>
       </c>
       <c r="F120" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="G120" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H120" s="1"/>
+      <c r="H120" s="1" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A121" s="3" t="s">
         <v>279</v>
       </c>
       <c r="B121" s="6" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="C121" s="1" t="s">
         <v>280</v>
@@ -4573,12 +4593,12 @@
         <v>51</v>
       </c>
       <c r="E121" s="5" t="s">
-        <v>270</v>
+        <v>226</v>
       </c>
       <c r="F121" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="G121" s="1" t="n">
+      <c r="H121" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4587,7 +4607,7 @@
         <v>281</v>
       </c>
       <c r="B122" s="6" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="C122" s="1" t="s">
         <v>282</v>
@@ -4596,7 +4616,7 @@
         <v>51</v>
       </c>
       <c r="E122" s="5" t="s">
-        <v>220</v>
+        <v>226</v>
       </c>
       <c r="F122" s="1" t="n">
         <v>0</v>
@@ -4610,7 +4630,7 @@
         <v>283</v>
       </c>
       <c r="B123" s="6" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="C123" s="1" t="s">
         <v>284</v>
@@ -4619,21 +4639,22 @@
         <v>51</v>
       </c>
       <c r="E123" s="5" t="s">
-        <v>220</v>
+        <v>254</v>
       </c>
       <c r="F123" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="H123" s="1" t="n">
-        <v>0</v>
-      </c>
+      <c r="G123" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H123" s="1"/>
     </row>
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A124" s="3" t="s">
         <v>285</v>
       </c>
       <c r="B124" s="6" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="C124" s="1" t="s">
         <v>286</v>
@@ -4642,12 +4663,12 @@
         <v>51</v>
       </c>
       <c r="E124" s="5" t="s">
-        <v>220</v>
+        <v>276</v>
       </c>
       <c r="F124" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="H124" s="1" t="n">
+      <c r="G124" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4656,7 +4677,7 @@
         <v>287</v>
       </c>
       <c r="B125" s="6" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="C125" s="1" t="s">
         <v>288</v>
@@ -4665,22 +4686,21 @@
         <v>51</v>
       </c>
       <c r="E125" s="5" t="s">
-        <v>248</v>
+        <v>226</v>
       </c>
       <c r="F125" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="G125" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H125" s="1"/>
+      <c r="H125" s="1" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A126" s="3" t="s">
         <v>289</v>
       </c>
       <c r="B126" s="6" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="C126" s="1" t="s">
         <v>290</v>
@@ -4688,54 +4708,54 @@
       <c r="D126" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="E126" s="9" t="s">
-        <v>291</v>
+      <c r="E126" s="5" t="s">
+        <v>226</v>
       </c>
       <c r="F126" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="G126" s="1" t="n">
+      <c r="H126" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A127" s="3" t="s">
+        <v>291</v>
+      </c>
+      <c r="B127" s="6" t="s">
+        <v>220</v>
+      </c>
+      <c r="C127" s="1" t="s">
         <v>292</v>
       </c>
-      <c r="B127" s="6" t="s">
-        <v>214</v>
-      </c>
-      <c r="C127" s="1" t="s">
-        <v>293</v>
-      </c>
       <c r="D127" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="E127" s="9" t="s">
-        <v>294</v>
+      <c r="E127" s="5" t="s">
+        <v>226</v>
       </c>
       <c r="F127" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="G127" s="1" t="n">
+      <c r="H127" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A128" s="3" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="B128" s="6" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="C128" s="1" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="D128" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="E128" s="1" t="s">
-        <v>297</v>
+      <c r="E128" s="5" t="s">
+        <v>254</v>
       </c>
       <c r="F128" s="1" t="n">
         <v>0</v>
@@ -4743,21 +4763,22 @@
       <c r="G128" s="1" t="n">
         <v>0</v>
       </c>
+      <c r="H128" s="1"/>
     </row>
     <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A129" s="3" t="s">
-        <v>298</v>
-      </c>
-      <c r="B129" s="3" t="s">
-        <v>299</v>
+        <v>295</v>
+      </c>
+      <c r="B129" s="6" t="s">
+        <v>220</v>
       </c>
       <c r="C129" s="1" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
       <c r="D129" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="E129" s="1" t="s">
+      <c r="E129" s="9" t="s">
         <v>297</v>
       </c>
       <c r="F129" s="1" t="n">
@@ -4769,19 +4790,19 @@
     </row>
     <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A130" s="3" t="s">
-        <v>301</v>
-      </c>
-      <c r="B130" s="3" t="s">
+        <v>298</v>
+      </c>
+      <c r="B130" s="6" t="s">
+        <v>220</v>
+      </c>
+      <c r="C130" s="1" t="s">
         <v>299</v>
       </c>
-      <c r="C130" s="1" t="s">
-        <v>302</v>
-      </c>
       <c r="D130" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="E130" s="1" t="s">
-        <v>297</v>
+      <c r="E130" s="9" t="s">
+        <v>300</v>
       </c>
       <c r="F130" s="1" t="n">
         <v>0</v>
@@ -4792,19 +4813,19 @@
     </row>
     <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A131" s="3" t="s">
+        <v>301</v>
+      </c>
+      <c r="B131" s="6" t="s">
+        <v>220</v>
+      </c>
+      <c r="C131" s="1" t="s">
+        <v>302</v>
+      </c>
+      <c r="D131" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E131" s="1" t="s">
         <v>303</v>
-      </c>
-      <c r="B131" s="3" t="s">
-        <v>299</v>
-      </c>
-      <c r="C131" s="1" t="s">
-        <v>304</v>
-      </c>
-      <c r="D131" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="E131" s="1" t="s">
-        <v>305</v>
       </c>
       <c r="F131" s="1" t="n">
         <v>0</v>
@@ -4815,19 +4836,19 @@
     </row>
     <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A132" s="3" t="s">
+        <v>304</v>
+      </c>
+      <c r="B132" s="3" t="s">
+        <v>305</v>
+      </c>
+      <c r="C132" s="1" t="s">
         <v>306</v>
       </c>
-      <c r="B132" s="3" t="s">
-        <v>299</v>
-      </c>
-      <c r="C132" s="1" t="s">
-        <v>307</v>
-      </c>
       <c r="D132" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="E132" s="7" t="s">
-        <v>308</v>
+      <c r="E132" s="1" t="s">
+        <v>303</v>
       </c>
       <c r="F132" s="1" t="n">
         <v>0</v>
@@ -4838,19 +4859,19 @@
     </row>
     <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A133" s="3" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="B133" s="3" t="s">
-        <v>299</v>
+        <v>305</v>
       </c>
       <c r="C133" s="1" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="D133" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="E133" s="7" t="s">
-        <v>308</v>
+      <c r="E133" s="1" t="s">
+        <v>303</v>
       </c>
       <c r="F133" s="1" t="n">
         <v>0</v>
@@ -4861,19 +4882,19 @@
     </row>
     <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A134" s="3" t="s">
+        <v>309</v>
+      </c>
+      <c r="B134" s="3" t="s">
+        <v>305</v>
+      </c>
+      <c r="C134" s="1" t="s">
+        <v>310</v>
+      </c>
+      <c r="D134" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E134" s="1" t="s">
         <v>311</v>
-      </c>
-      <c r="B134" s="3" t="s">
-        <v>299</v>
-      </c>
-      <c r="C134" s="1" t="s">
-        <v>312</v>
-      </c>
-      <c r="D134" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="E134" s="7" t="s">
-        <v>308</v>
       </c>
       <c r="F134" s="1" t="n">
         <v>0</v>
@@ -4884,19 +4905,19 @@
     </row>
     <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A135" s="3" t="s">
+        <v>312</v>
+      </c>
+      <c r="B135" s="3" t="s">
+        <v>305</v>
+      </c>
+      <c r="C135" s="1" t="s">
         <v>313</v>
       </c>
-      <c r="B135" s="3" t="s">
-        <v>299</v>
-      </c>
-      <c r="C135" s="1" t="s">
+      <c r="D135" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E135" s="7" t="s">
         <v>314</v>
-      </c>
-      <c r="D135" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="E135" s="7" t="s">
-        <v>315</v>
       </c>
       <c r="F135" s="1" t="n">
         <v>0</v>
@@ -4907,19 +4928,19 @@
     </row>
     <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A136" s="3" t="s">
+        <v>315</v>
+      </c>
+      <c r="B136" s="3" t="s">
+        <v>305</v>
+      </c>
+      <c r="C136" s="1" t="s">
         <v>316</v>
       </c>
-      <c r="B136" s="3" t="s">
-        <v>299</v>
-      </c>
-      <c r="C136" s="1" t="s">
-        <v>317</v>
-      </c>
       <c r="D136" s="1" t="s">
         <v>51</v>
       </c>
       <c r="E136" s="7" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="F136" s="1" t="n">
         <v>0</v>
@@ -4930,19 +4951,19 @@
     </row>
     <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A137" s="3" t="s">
+        <v>317</v>
+      </c>
+      <c r="B137" s="3" t="s">
+        <v>305</v>
+      </c>
+      <c r="C137" s="1" t="s">
         <v>318</v>
       </c>
-      <c r="B137" s="3" t="s">
-        <v>299</v>
-      </c>
-      <c r="C137" s="1" t="s">
-        <v>319</v>
-      </c>
       <c r="D137" s="1" t="s">
         <v>51</v>
       </c>
       <c r="E137" s="7" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="F137" s="1" t="n">
         <v>0</v>
@@ -4953,19 +4974,19 @@
     </row>
     <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A138" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="B138" s="3" t="s">
+        <v>305</v>
+      </c>
+      <c r="C138" s="1" t="s">
         <v>320</v>
       </c>
-      <c r="B138" s="3" t="s">
-        <v>299</v>
-      </c>
-      <c r="C138" s="1" t="s">
+      <c r="D138" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E138" s="7" t="s">
         <v>321</v>
-      </c>
-      <c r="D138" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="E138" s="7" t="s">
-        <v>322</v>
       </c>
       <c r="F138" s="1" t="n">
         <v>0</v>
@@ -4976,19 +4997,19 @@
     </row>
     <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A139" s="3" t="s">
+        <v>322</v>
+      </c>
+      <c r="B139" s="3" t="s">
+        <v>305</v>
+      </c>
+      <c r="C139" s="1" t="s">
         <v>323</v>
       </c>
-      <c r="B139" s="3" t="s">
-        <v>299</v>
-      </c>
-      <c r="C139" s="1" t="s">
-        <v>324</v>
-      </c>
       <c r="D139" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="E139" s="1" t="s">
-        <v>325</v>
+      <c r="E139" s="7" t="s">
+        <v>321</v>
       </c>
       <c r="F139" s="1" t="n">
         <v>0</v>
@@ -4999,19 +5020,19 @@
     </row>
     <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A140" s="3" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="B140" s="3" t="s">
-        <v>299</v>
+        <v>305</v>
       </c>
       <c r="C140" s="1" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="D140" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="E140" s="1" t="s">
-        <v>328</v>
+      <c r="E140" s="7" t="s">
+        <v>321</v>
       </c>
       <c r="F140" s="1" t="n">
         <v>0</v>
@@ -5022,19 +5043,19 @@
     </row>
     <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A141" s="3" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
       <c r="B141" s="3" t="s">
-        <v>299</v>
+        <v>305</v>
       </c>
       <c r="C141" s="1" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
       <c r="D141" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="E141" s="1" t="s">
-        <v>331</v>
+      <c r="E141" s="7" t="s">
+        <v>328</v>
       </c>
       <c r="F141" s="1" t="n">
         <v>0</v>
@@ -5045,19 +5066,19 @@
     </row>
     <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A142" s="3" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
       <c r="B142" s="3" t="s">
-        <v>299</v>
+        <v>305</v>
       </c>
       <c r="C142" s="1" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
       <c r="D142" s="1" t="s">
         <v>51</v>
       </c>
       <c r="E142" s="1" t="s">
-        <v>334</v>
+        <v>331</v>
       </c>
       <c r="F142" s="1" t="n">
         <v>0</v>
@@ -5068,19 +5089,19 @@
     </row>
     <row r="143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A143" s="3" t="s">
-        <v>335</v>
+        <v>332</v>
       </c>
       <c r="B143" s="3" t="s">
-        <v>299</v>
+        <v>305</v>
       </c>
       <c r="C143" s="1" t="s">
-        <v>336</v>
+        <v>333</v>
       </c>
       <c r="D143" s="1" t="s">
         <v>51</v>
       </c>
       <c r="E143" s="1" t="s">
-        <v>337</v>
+        <v>334</v>
       </c>
       <c r="F143" s="1" t="n">
         <v>0</v>
@@ -5091,13 +5112,13 @@
     </row>
     <row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A144" s="3" t="s">
-        <v>338</v>
+        <v>335</v>
       </c>
       <c r="B144" s="3" t="s">
-        <v>299</v>
+        <v>305</v>
       </c>
       <c r="C144" s="1" t="s">
-        <v>339</v>
+        <v>336</v>
       </c>
       <c r="D144" s="1" t="s">
         <v>51</v>
@@ -5114,45 +5135,42 @@
     </row>
     <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A145" s="3" t="s">
+        <v>338</v>
+      </c>
+      <c r="B145" s="3" t="s">
+        <v>305</v>
+      </c>
+      <c r="C145" s="1" t="s">
+        <v>339</v>
+      </c>
+      <c r="D145" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E145" s="1" t="s">
         <v>340</v>
       </c>
-      <c r="B145" s="3" t="s">
-        <v>299</v>
-      </c>
-      <c r="C145" s="1" t="s">
-        <v>341</v>
-      </c>
-      <c r="D145" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="E145" s="1" t="s">
-        <v>78</v>
-      </c>
       <c r="F145" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G145" s="1" t="n">
         <v>0</v>
-      </c>
-      <c r="H145" s="1" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A146" s="3" t="s">
+        <v>341</v>
+      </c>
+      <c r="B146" s="3" t="s">
+        <v>305</v>
+      </c>
+      <c r="C146" s="1" t="s">
         <v>342</v>
       </c>
-      <c r="B146" s="3" t="s">
+      <c r="D146" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E146" s="1" t="s">
         <v>343</v>
-      </c>
-      <c r="C146" s="1" t="s">
-        <v>344</v>
-      </c>
-      <c r="D146" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="E146" s="1" t="s">
-        <v>345</v>
       </c>
       <c r="F146" s="1" t="n">
         <v>0</v>
@@ -5163,19 +5181,19 @@
     </row>
     <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A147" s="3" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="B147" s="3" t="s">
+        <v>305</v>
+      </c>
+      <c r="C147" s="1" t="s">
+        <v>345</v>
+      </c>
+      <c r="D147" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E147" s="1" t="s">
         <v>343</v>
-      </c>
-      <c r="C147" s="1" t="s">
-        <v>347</v>
-      </c>
-      <c r="D147" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="E147" s="1" t="s">
-        <v>348</v>
       </c>
       <c r="F147" s="1" t="n">
         <v>0</v>
@@ -5186,145 +5204,148 @@
     </row>
     <row r="148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A148" s="3" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="B148" s="3" t="s">
-        <v>343</v>
+        <v>305</v>
       </c>
       <c r="C148" s="1" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
       <c r="D148" s="1" t="s">
         <v>51</v>
       </c>
+      <c r="E148" s="1" t="s">
+        <v>78</v>
+      </c>
       <c r="F148" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="G148" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H148" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="149" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A149" s="3" t="s">
+        <v>348</v>
+      </c>
+      <c r="B149" s="3" t="s">
+        <v>349</v>
+      </c>
+      <c r="C149" s="1" t="s">
+        <v>350</v>
+      </c>
+      <c r="D149" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E149" s="1" t="s">
         <v>351</v>
       </c>
-      <c r="B149" s="3" t="s">
-        <v>343</v>
-      </c>
-      <c r="C149" s="1" t="s">
+      <c r="F149" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G149" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="150" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A150" s="3" t="s">
         <v>352</v>
       </c>
-      <c r="D149" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="F149" s="1" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="150" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A150" s="7" t="s">
+      <c r="B150" s="3" t="s">
+        <v>349</v>
+      </c>
+      <c r="C150" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="B150" s="7" t="s">
+      <c r="D150" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E150" s="1" t="s">
         <v>354</v>
       </c>
-      <c r="C150" s="1" t="s">
+      <c r="F150" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G150" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="151" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A151" s="3" t="s">
         <v>355</v>
       </c>
-      <c r="D150" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="E150" s="1" t="s">
+      <c r="B151" s="3" t="s">
+        <v>349</v>
+      </c>
+      <c r="C151" s="1" t="s">
+        <v>356</v>
+      </c>
+      <c r="D151" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="F151" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="152" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A152" s="3" t="s">
+        <v>357</v>
+      </c>
+      <c r="B152" s="3" t="s">
+        <v>349</v>
+      </c>
+      <c r="C152" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="D152" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="F152" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="153" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A153" s="7" t="s">
+        <v>359</v>
+      </c>
+      <c r="B153" s="7" t="s">
+        <v>360</v>
+      </c>
+      <c r="C153" s="1" t="s">
+        <v>361</v>
+      </c>
+      <c r="D153" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E153" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="F150" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G150" s="1" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="151" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A151" s="7" t="s">
-        <v>356</v>
-      </c>
-      <c r="B151" s="7" t="s">
-        <v>354</v>
-      </c>
-      <c r="C151" s="1" t="s">
-        <v>357</v>
-      </c>
-      <c r="D151" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="E151" s="1" t="s">
+      <c r="F153" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G153" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="154" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A154" s="7" t="s">
+        <v>362</v>
+      </c>
+      <c r="B154" s="7" t="s">
+        <v>360</v>
+      </c>
+      <c r="C154" s="1" t="s">
+        <v>363</v>
+      </c>
+      <c r="D154" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E154" s="1" t="s">
         <v>52</v>
-      </c>
-      <c r="F151" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G151" s="1" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="152" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A152" s="1" t="s">
-        <v>358</v>
-      </c>
-      <c r="B152" s="7" t="s">
-        <v>354</v>
-      </c>
-      <c r="C152" s="1" t="s">
-        <v>359</v>
-      </c>
-      <c r="D152" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="E152" s="1" t="s">
-        <v>360</v>
-      </c>
-      <c r="F152" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G152" s="1" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="153" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A153" s="1" t="s">
-        <v>361</v>
-      </c>
-      <c r="B153" s="7" t="s">
-        <v>354</v>
-      </c>
-      <c r="C153" s="1" t="s">
-        <v>362</v>
-      </c>
-      <c r="D153" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="E153" s="1" t="s">
-        <v>363</v>
-      </c>
-      <c r="F153" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G153" s="1" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="154" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A154" s="1" t="s">
-        <v>364</v>
-      </c>
-      <c r="B154" s="7" t="s">
-        <v>354</v>
-      </c>
-      <c r="C154" s="1" t="s">
-        <v>365</v>
-      </c>
-      <c r="D154" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="E154" s="1" t="s">
-        <v>366</v>
       </c>
       <c r="F154" s="1" t="n">
         <v>0</v>
@@ -5335,64 +5356,70 @@
     </row>
     <row r="155" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A155" s="1" t="s">
+        <v>364</v>
+      </c>
+      <c r="B155" s="7" t="s">
+        <v>360</v>
+      </c>
+      <c r="C155" s="1" t="s">
+        <v>365</v>
+      </c>
+      <c r="D155" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E155" s="1" t="s">
+        <v>366</v>
+      </c>
+      <c r="F155" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G155" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="156" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A156" s="1" t="s">
         <v>367</v>
       </c>
-      <c r="B155" s="7" t="s">
-        <v>354</v>
-      </c>
-      <c r="C155" s="1" t="s">
+      <c r="B156" s="7" t="s">
+        <v>360</v>
+      </c>
+      <c r="C156" s="1" t="s">
         <v>368</v>
       </c>
-      <c r="D155" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="F155" s="1" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="156" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A156" s="7" t="s">
+      <c r="D156" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E156" s="1" t="s">
         <v>369</v>
       </c>
-      <c r="B156" s="7" t="s">
-        <v>354</v>
-      </c>
-      <c r="C156" s="1" t="s">
-        <v>370</v>
-      </c>
-      <c r="D156" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="E156" s="1" t="s">
-        <v>78</v>
-      </c>
       <c r="F156" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G156" s="1" t="n">
         <v>0</v>
-      </c>
-      <c r="H156" s="1" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="157" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A157" s="1" t="s">
+        <v>370</v>
+      </c>
+      <c r="B157" s="7" t="s">
+        <v>360</v>
+      </c>
+      <c r="C157" s="1" t="s">
         <v>371</v>
       </c>
-      <c r="B157" s="7" t="s">
-        <v>354</v>
-      </c>
-      <c r="C157" s="1" t="s">
+      <c r="D157" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E157" s="1" t="s">
         <v>372</v>
       </c>
-      <c r="D157" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="E157" s="1" t="s">
-        <v>110</v>
-      </c>
       <c r="F157" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G157" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5401,7 +5428,7 @@
         <v>373</v>
       </c>
       <c r="B158" s="7" t="s">
-        <v>354</v>
+        <v>360</v>
       </c>
       <c r="C158" s="1" t="s">
         <v>374</v>
@@ -5409,22 +5436,16 @@
       <c r="D158" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="E158" s="1" t="s">
-        <v>205</v>
-      </c>
       <c r="F158" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="G158" s="1" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="159" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A159" s="1" t="s">
+      <c r="A159" s="7" t="s">
         <v>375</v>
       </c>
       <c r="B159" s="7" t="s">
-        <v>354</v>
+        <v>360</v>
       </c>
       <c r="C159" s="1" t="s">
         <v>376</v>
@@ -5433,7 +5454,7 @@
         <v>51</v>
       </c>
       <c r="E159" s="1" t="s">
-        <v>164</v>
+        <v>78</v>
       </c>
       <c r="F159" s="1" t="n">
         <v>0</v>
@@ -5442,15 +5463,15 @@
         <v>0</v>
       </c>
       <c r="H159" s="1" t="n">
-        <v>100</v>
+        <v>1</v>
       </c>
     </row>
     <row r="160" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A160" s="1" t="s">
         <v>377</v>
       </c>
-      <c r="B160" s="1" t="s">
-        <v>354</v>
+      <c r="B160" s="7" t="s">
+        <v>360</v>
       </c>
       <c r="C160" s="1" t="s">
         <v>378</v>
@@ -5459,12 +5480,9 @@
         <v>51</v>
       </c>
       <c r="E160" s="1" t="s">
-        <v>363</v>
+        <v>110</v>
       </c>
       <c r="F160" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G160" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5472,8 +5490,8 @@
       <c r="A161" s="1" t="s">
         <v>379</v>
       </c>
-      <c r="B161" s="1" t="s">
-        <v>354</v>
+      <c r="B161" s="7" t="s">
+        <v>360</v>
       </c>
       <c r="C161" s="1" t="s">
         <v>380</v>
@@ -5482,7 +5500,7 @@
         <v>51</v>
       </c>
       <c r="E161" s="1" t="s">
-        <v>52</v>
+        <v>211</v>
       </c>
       <c r="F161" s="1" t="n">
         <v>0</v>
@@ -5496,7 +5514,7 @@
         <v>381</v>
       </c>
       <c r="B162" s="7" t="s">
-        <v>354</v>
+        <v>360</v>
       </c>
       <c r="C162" s="1" t="s">
         <v>382</v>
@@ -5505,21 +5523,24 @@
         <v>51</v>
       </c>
       <c r="E162" s="1" t="s">
-        <v>52</v>
+        <v>170</v>
       </c>
       <c r="F162" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G162" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="H162" s="1" t="n">
+        <v>100</v>
       </c>
     </row>
     <row r="163" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A163" s="1" t="s">
         <v>383</v>
       </c>
-      <c r="B163" s="7" t="s">
-        <v>354</v>
+      <c r="B163" s="1" t="s">
+        <v>360</v>
       </c>
       <c r="C163" s="1" t="s">
         <v>384</v>
@@ -5528,7 +5549,7 @@
         <v>51</v>
       </c>
       <c r="E163" s="1" t="s">
-        <v>52</v>
+        <v>369</v>
       </c>
       <c r="F163" s="1" t="n">
         <v>0</v>
@@ -5541,8 +5562,8 @@
       <c r="A164" s="1" t="s">
         <v>385</v>
       </c>
-      <c r="B164" s="7" t="s">
-        <v>354</v>
+      <c r="B164" s="1" t="s">
+        <v>360</v>
       </c>
       <c r="C164" s="1" t="s">
         <v>386</v>
@@ -5551,7 +5572,7 @@
         <v>51</v>
       </c>
       <c r="E164" s="1" t="s">
-        <v>387</v>
+        <v>52</v>
       </c>
       <c r="F164" s="1" t="n">
         <v>0</v>
@@ -5562,80 +5583,71 @@
     </row>
     <row r="165" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A165" s="1" t="s">
+        <v>387</v>
+      </c>
+      <c r="B165" s="7" t="s">
+        <v>360</v>
+      </c>
+      <c r="C165" s="1" t="s">
         <v>388</v>
       </c>
-      <c r="B165" s="7" t="s">
-        <v>354</v>
-      </c>
-      <c r="C165" s="1" t="s">
-        <v>389</v>
-      </c>
       <c r="D165" s="1" t="s">
         <v>51</v>
       </c>
       <c r="E165" s="1" t="s">
-        <v>164</v>
+        <v>52</v>
       </c>
       <c r="F165" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G165" s="1" t="n">
         <v>0</v>
-      </c>
-      <c r="H165" s="1" t="n">
-        <v>100</v>
       </c>
     </row>
     <row r="166" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A166" s="1" t="s">
+        <v>389</v>
+      </c>
+      <c r="B166" s="7" t="s">
+        <v>360</v>
+      </c>
+      <c r="C166" s="1" t="s">
         <v>390</v>
       </c>
-      <c r="B166" s="7" t="s">
-        <v>354</v>
-      </c>
-      <c r="C166" s="1" t="s">
-        <v>391</v>
-      </c>
       <c r="D166" s="1" t="s">
         <v>51</v>
       </c>
       <c r="E166" s="1" t="s">
-        <v>78</v>
+        <v>52</v>
       </c>
       <c r="F166" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G166" s="1" t="n">
         <v>0</v>
-      </c>
-      <c r="H166" s="1" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="167" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A167" s="1" t="s">
+        <v>391</v>
+      </c>
+      <c r="B167" s="7" t="s">
+        <v>360</v>
+      </c>
+      <c r="C167" s="1" t="s">
         <v>392</v>
       </c>
-      <c r="B167" s="7" t="s">
-        <v>354</v>
-      </c>
-      <c r="C167" s="7" t="s">
+      <c r="D167" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E167" s="1" t="s">
         <v>393</v>
       </c>
-      <c r="D167" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="E167" s="1" t="s">
-        <v>78</v>
-      </c>
       <c r="F167" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G167" s="1" t="n">
         <v>0</v>
-      </c>
-      <c r="H167" s="1" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="168" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5643,16 +5655,16 @@
         <v>394</v>
       </c>
       <c r="B168" s="7" t="s">
-        <v>354</v>
-      </c>
-      <c r="C168" s="7" t="s">
+        <v>360</v>
+      </c>
+      <c r="C168" s="1" t="s">
         <v>395</v>
       </c>
       <c r="D168" s="1" t="s">
         <v>51</v>
       </c>
       <c r="E168" s="1" t="s">
-        <v>78</v>
+        <v>170</v>
       </c>
       <c r="F168" s="1" t="n">
         <v>0</v>
@@ -5661,7 +5673,7 @@
         <v>0</v>
       </c>
       <c r="H168" s="1" t="n">
-        <v>1</v>
+        <v>100</v>
       </c>
     </row>
     <row r="169" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5669,7 +5681,7 @@
         <v>396</v>
       </c>
       <c r="B169" s="7" t="s">
-        <v>354</v>
+        <v>360</v>
       </c>
       <c r="C169" s="1" t="s">
         <v>397</v>
@@ -5678,13 +5690,16 @@
         <v>51</v>
       </c>
       <c r="E169" s="1" t="s">
-        <v>387</v>
+        <v>78</v>
       </c>
       <c r="F169" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G169" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="H169" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="170" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5692,21 +5707,96 @@
         <v>398</v>
       </c>
       <c r="B170" s="7" t="s">
-        <v>354</v>
-      </c>
-      <c r="C170" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="C170" s="7" t="s">
         <v>399</v>
       </c>
       <c r="D170" s="1" t="s">
         <v>51</v>
       </c>
       <c r="E170" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="F170" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G170" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H170" s="1" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="171" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A171" s="1" t="s">
+        <v>400</v>
+      </c>
+      <c r="B171" s="7" t="s">
+        <v>360</v>
+      </c>
+      <c r="C171" s="7" t="s">
+        <v>401</v>
+      </c>
+      <c r="D171" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E171" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="F171" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G171" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H171" s="1" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="172" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A172" s="1" t="s">
+        <v>402</v>
+      </c>
+      <c r="B172" s="7" t="s">
+        <v>360</v>
+      </c>
+      <c r="C172" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="D172" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E172" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="F172" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G172" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="173" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A173" s="1" t="s">
+        <v>404</v>
+      </c>
+      <c r="B173" s="7" t="s">
+        <v>360</v>
+      </c>
+      <c r="C173" s="1" t="s">
+        <v>405</v>
+      </c>
+      <c r="D173" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E173" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="F170" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G170" s="1" t="n">
+      <c r="F173" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G173" s="1" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>